<commit_message>
Checkpoint sebelum running ulang perbaikan Turn Penalty untuk loncatan
</commit_message>
<xml_diff>
--- a/Excel/Rekap/Avg_Keseluruhan_All.xlsx
+++ b/Excel/Rekap/Avg_Keseluruhan_All.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEMHAS\TA_Python_Server\Excel\Rekap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB5B2CA-FE1E-4587-AE15-74E1A2A098AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70FFAE1F-FC6A-40D5-BC1F-A73F9132D108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -334,7 +334,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -683,157 +683,157 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="B2">
-        <v>5.4570399999999989E-3</v>
+        <v>4.1219049999999986E-3</v>
       </c>
       <c r="C2">
-        <v>92.764815679459943</v>
+        <v>97.253304076183326</v>
       </c>
       <c r="D2">
-        <v>16.75</v>
+        <v>11.75</v>
       </c>
       <c r="E2">
-        <v>35.049999999999997</v>
+        <v>26.95</v>
       </c>
       <c r="F2">
-        <v>7.2</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>26.82837878657665</v>
+        <v>25.99290433019722</v>
       </c>
       <c r="H2">
         <f>_xlfn.VAR.S(B2:F2)</f>
-        <v>1389.843230388904</v>
+        <v>1550.2597753266573</v>
       </c>
       <c r="I2">
         <f>_xlfn.STDEV.S(B2:F2)</f>
-        <v>37.280601261096955</v>
+        <v>39.373338381786439</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="B3">
-        <v>5.3549600000000006E-3</v>
+        <v>4.2538850000000007E-3</v>
       </c>
       <c r="C3">
-        <v>95.466460966906681</v>
+        <v>97.253304076183326</v>
       </c>
       <c r="D3">
-        <v>16.75</v>
+        <v>11.65</v>
       </c>
       <c r="E3">
-        <v>35.049999999999997</v>
+        <v>27.55</v>
       </c>
       <c r="F3">
-        <v>9.0500000000000007</v>
+        <v>9</v>
       </c>
       <c r="G3">
-        <v>29.061969321151121</v>
+        <v>26.07625966019722</v>
       </c>
       <c r="H3">
         <f>_xlfn.VAR.S(B3:F3)</f>
-        <v>1454.3776678210934</v>
+        <v>1550.5874845559779</v>
       </c>
       <c r="I3">
         <f>_xlfn.STDEV.S(B3:F3)</f>
-        <v>38.136303803870312</v>
+        <v>39.377499724537842</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="B4">
-        <v>6.0128149999999986E-3</v>
+        <v>4.4020500000000002E-3</v>
       </c>
       <c r="C4">
-        <v>95.679034212460891</v>
+        <v>97.581102103629476</v>
       </c>
       <c r="D4">
-        <v>17.45</v>
+        <v>12.45</v>
       </c>
       <c r="E4">
-        <v>33.4</v>
+        <v>27.75</v>
       </c>
       <c r="F4">
-        <v>8.9</v>
+        <v>9.4</v>
       </c>
       <c r="G4">
-        <v>27.73084117124348</v>
+        <v>26.430917358938249</v>
       </c>
       <c r="H4">
         <f>_xlfn.VAR.S(B4:F4)</f>
-        <v>1455.4348387743521</v>
+        <v>1550.6954951363477</v>
       </c>
       <c r="I4">
         <f>_xlfn.STDEV.S(B4:F4)</f>
-        <v>38.150161713606828</v>
+        <v>39.378871176512256</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="B5">
-        <v>6.3522550000000011E-3</v>
+        <v>4.4211700000000003E-3</v>
       </c>
       <c r="C5">
-        <v>94.324349526678361</v>
+        <v>97.581102103629476</v>
       </c>
       <c r="D5">
-        <v>15</v>
+        <v>12.45</v>
       </c>
       <c r="E5">
-        <v>41.8</v>
+        <v>27.75</v>
       </c>
       <c r="F5">
-        <v>7.95</v>
+        <v>9.4</v>
       </c>
       <c r="G5">
-        <v>28.17178363027972</v>
+        <v>26.43092054560492</v>
       </c>
       <c r="H5">
         <f>_xlfn.VAR.S(B5:F5)</f>
-        <v>1467.7978795279689</v>
+        <v>1550.6952137598203</v>
       </c>
       <c r="I5">
         <f>_xlfn.STDEV.S(B5:F5)</f>
-        <v>38.311850379849432</v>
+        <v>39.378867603828077</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="B6">
-        <v>5.0669699999999996E-3</v>
+        <v>5.4570399999999989E-3</v>
       </c>
       <c r="C6">
-        <v>96.40095104720146</v>
+        <v>92.764815679459943</v>
       </c>
       <c r="D6">
-        <v>17.399999999999999</v>
+        <v>16.75</v>
       </c>
       <c r="E6">
-        <v>30.85</v>
+        <v>35.049999999999997</v>
       </c>
       <c r="F6">
-        <v>9.15</v>
+        <v>7.2</v>
       </c>
       <c r="G6">
-        <v>27.509336336200249</v>
+        <v>26.82837878657665</v>
       </c>
       <c r="H6">
         <f>_xlfn.VAR.S(B6:F6)</f>
-        <v>1475.0225382043941</v>
+        <v>1389.843230388904</v>
       </c>
       <c r="I6">
         <f>_xlfn.STDEV.S(B6:F6)</f>
-        <v>38.406022160650721</v>
+        <v>37.280601261096955</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -900,261 +900,261 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B9">
-        <v>6.5454250000000014E-3</v>
+        <v>5.0669699999999996E-3</v>
       </c>
       <c r="C9">
-        <v>95.302702649425811</v>
+        <v>96.40095104720146</v>
       </c>
       <c r="D9">
-        <v>14.75</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="E9">
-        <v>42.05</v>
+        <v>30.85</v>
       </c>
       <c r="F9">
-        <v>8.5</v>
+        <v>9.15</v>
       </c>
       <c r="G9">
-        <v>28.518208012404301</v>
+        <v>27.509336336200249</v>
       </c>
       <c r="H9">
         <f>_xlfn.VAR.S(B9:F9)</f>
-        <v>1495.3885154302432</v>
+        <v>1475.0225382043941</v>
       </c>
       <c r="I9">
         <f>_xlfn.STDEV.S(B9:F9)</f>
-        <v>38.670253625108835</v>
+        <v>38.406022160650721</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="B10">
-        <v>6.2702000000000009E-3</v>
+        <v>5.3969999999999999E-3</v>
       </c>
       <c r="C10">
-        <v>95.905800795126837</v>
+        <v>99.522392368525942</v>
       </c>
       <c r="D10">
-        <v>15</v>
+        <v>16.95</v>
       </c>
       <c r="E10">
-        <v>41.8</v>
+        <v>32</v>
       </c>
       <c r="F10">
-        <v>9.6</v>
+        <v>7.75</v>
       </c>
       <c r="G10">
-        <v>29.993678499187801</v>
+        <v>27.662964894754321</v>
       </c>
       <c r="H10">
         <f>_xlfn.VAR.S(B10:F10)</f>
-        <v>1498.3202468311349</v>
+        <v>1598.6617944217842</v>
       </c>
       <c r="I10">
         <f>_xlfn.STDEV.S(B10:F10)</f>
-        <v>38.708141867456447</v>
+        <v>39.983268931163998</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
       <c r="B11">
-        <v>7.9057550000000004E-3</v>
+        <v>6.0128149999999986E-3</v>
       </c>
       <c r="C11">
-        <v>94.129850728560768</v>
+        <v>95.679034212460891</v>
       </c>
       <c r="D11">
-        <v>12.25</v>
+        <v>17.45</v>
       </c>
       <c r="E11">
-        <v>46.65</v>
+        <v>33.4</v>
       </c>
       <c r="F11">
-        <v>7</v>
+        <v>8.9</v>
       </c>
       <c r="G11">
-        <v>28.17295941392679</v>
+        <v>27.73084117124348</v>
       </c>
       <c r="H11">
         <f>_xlfn.VAR.S(B11:F11)</f>
-        <v>1528.3242901559486</v>
+        <v>1455.4348387743521</v>
       </c>
       <c r="I11">
         <f>_xlfn.STDEV.S(B11:F11)</f>
-        <v>39.09378838327067</v>
+        <v>38.150161713606828</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B12">
-        <v>6.4687750000000004E-3</v>
+        <v>4.0263149999999999E-3</v>
       </c>
       <c r="C12">
-        <v>97.195750288788005</v>
+        <v>99.130927060973946</v>
       </c>
       <c r="D12">
-        <v>14.75</v>
+        <v>11.75</v>
       </c>
       <c r="E12">
-        <v>42.05</v>
+        <v>26.95</v>
       </c>
       <c r="F12">
-        <v>10.25</v>
+        <v>10.85</v>
       </c>
       <c r="G12">
-        <v>30.483703177298</v>
+        <v>27.922492229328981</v>
       </c>
       <c r="H12">
         <f>_xlfn.VAR.S(B12:F12)</f>
-        <v>1535.5207806424405</v>
+        <v>1596.8962860240595</v>
       </c>
       <c r="I12">
         <f>_xlfn.STDEV.S(B12:F12)</f>
-        <v>39.18572164248657</v>
+        <v>39.961184742498055</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="B13">
-        <v>4.9714599999999996E-3</v>
+        <v>4.175425E-3</v>
       </c>
       <c r="C13">
-        <v>99.055191129685852</v>
+        <v>99.130927060973946</v>
       </c>
       <c r="D13">
-        <v>17.399999999999999</v>
+        <v>11.65</v>
       </c>
       <c r="E13">
-        <v>30.85</v>
+        <v>27.55</v>
       </c>
       <c r="F13">
-        <v>11.5</v>
+        <v>10.85</v>
       </c>
       <c r="G13">
-        <v>29.67669376494764</v>
+        <v>28.005850414328989</v>
       </c>
       <c r="H13">
         <f>_xlfn.VAR.S(B13:F13)</f>
-        <v>1538.6324665253799</v>
+        <v>1597.0373141630498</v>
       </c>
       <c r="I13">
         <f>_xlfn.STDEV.S(B13:F13)</f>
-        <v>39.225405880951442</v>
+        <v>39.962949267578459</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="B14">
-        <v>7.7220349999999986E-3</v>
+        <v>5.7693950000000009E-3</v>
       </c>
       <c r="C14">
-        <v>95.244064290933849</v>
+        <v>99.450828686644769</v>
       </c>
       <c r="D14">
-        <v>12.7</v>
+        <v>17</v>
       </c>
       <c r="E14">
-        <v>46</v>
+        <v>31.1</v>
       </c>
       <c r="F14">
-        <v>7.7</v>
+        <v>9.35</v>
       </c>
       <c r="G14">
-        <v>28.558631054322309</v>
+        <v>28.05109968027412</v>
       </c>
       <c r="H14">
         <f>_xlfn.VAR.S(B14:F14)</f>
-        <v>1545.4379594530731</v>
+        <v>1577.5409388588309</v>
       </c>
       <c r="I14">
         <f>_xlfn.STDEV.S(B14:F14)</f>
-        <v>39.312058702808649</v>
+        <v>39.71826958540403</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="B15">
-        <v>4.1219049999999986E-3</v>
+        <v>6.3522550000000011E-3</v>
       </c>
       <c r="C15">
-        <v>97.253304076183326</v>
+        <v>94.324349526678361</v>
       </c>
       <c r="D15">
-        <v>11.75</v>
+        <v>15</v>
       </c>
       <c r="E15">
-        <v>26.95</v>
+        <v>41.8</v>
       </c>
       <c r="F15">
-        <v>9</v>
+        <v>7.95</v>
       </c>
       <c r="G15">
-        <v>25.99290433019722</v>
+        <v>28.17178363027972</v>
       </c>
       <c r="H15">
         <f>_xlfn.VAR.S(B15:F15)</f>
-        <v>1550.2597753266573</v>
+        <v>1467.7978795279689</v>
       </c>
       <c r="I15">
         <f>_xlfn.STDEV.S(B15:F15)</f>
-        <v>39.373338381786439</v>
+        <v>38.311850379849432</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="B16">
-        <v>4.2538850000000007E-3</v>
+        <v>7.9057550000000004E-3</v>
       </c>
       <c r="C16">
-        <v>97.253304076183326</v>
+        <v>94.129850728560768</v>
       </c>
       <c r="D16">
-        <v>11.65</v>
+        <v>12.25</v>
       </c>
       <c r="E16">
-        <v>27.55</v>
+        <v>46.65</v>
       </c>
       <c r="F16">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G16">
-        <v>26.07625966019722</v>
+        <v>28.17295941392679</v>
       </c>
       <c r="H16">
         <f>_xlfn.VAR.S(B16:F16)</f>
-        <v>1550.5874845559779</v>
+        <v>1528.3242901559486</v>
       </c>
       <c r="I16">
         <f>_xlfn.STDEV.S(B16:F16)</f>
-        <v>39.377499724537842</v>
+        <v>39.09378838327067</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="B17">
-        <v>4.4211700000000003E-3</v>
+        <v>4.3084050000000004E-3</v>
       </c>
       <c r="C17">
-        <v>97.581102103629476</v>
+        <v>99.4652416360247</v>
       </c>
       <c r="D17">
         <v>12.45</v>
@@ -1163,29 +1163,29 @@
         <v>27.75</v>
       </c>
       <c r="F17">
-        <v>9.4</v>
+        <v>11.2</v>
       </c>
       <c r="G17">
-        <v>26.43092054560492</v>
+        <v>28.378258340170781</v>
       </c>
       <c r="H17">
         <f>_xlfn.VAR.S(B17:F17)</f>
-        <v>1550.6952137598203</v>
+        <v>1597.8787715897215</v>
       </c>
       <c r="I17">
         <f>_xlfn.STDEV.S(B17:F17)</f>
-        <v>39.378867603828077</v>
+        <v>39.973475850740343</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B18">
-        <v>4.4020500000000002E-3</v>
+        <v>4.3338500000000002E-3</v>
       </c>
       <c r="C18">
-        <v>97.581102103629476</v>
+        <v>99.4652416360247</v>
       </c>
       <c r="D18">
         <v>12.45</v>
@@ -1194,80 +1194,80 @@
         <v>27.75</v>
       </c>
       <c r="F18">
-        <v>9.4</v>
+        <v>11.2</v>
       </c>
       <c r="G18">
-        <v>26.430917358938249</v>
+        <v>28.378262581004108</v>
       </c>
       <c r="H18">
         <f>_xlfn.VAR.S(B18:F18)</f>
-        <v>1550.6954951363477</v>
+        <v>1597.8783877570943</v>
       </c>
       <c r="I18">
         <f>_xlfn.STDEV.S(B18:F18)</f>
-        <v>39.378871176512256</v>
+        <v>39.973471049648595</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>63</v>
       </c>
       <c r="B19">
-        <v>7.8221300000000001E-3</v>
+        <v>6.5454250000000014E-3</v>
       </c>
       <c r="C19">
-        <v>95.466460966906681</v>
+        <v>95.302702649425811</v>
       </c>
       <c r="D19">
-        <v>12.25</v>
+        <v>14.75</v>
       </c>
       <c r="E19">
-        <v>46.65</v>
+        <v>42.05</v>
       </c>
       <c r="F19">
         <v>8.5</v>
       </c>
       <c r="G19">
-        <v>30.004047182817779</v>
+        <v>28.518208012404301</v>
       </c>
       <c r="H19">
         <f>_xlfn.VAR.S(B19:F19)</f>
-        <v>1551.6934529663436</v>
+        <v>1495.3885154302432</v>
       </c>
       <c r="I19">
         <f>_xlfn.STDEV.S(B19:F19)</f>
-        <v>39.391540373109855</v>
+        <v>38.670253625108835</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B20">
-        <v>5.0783499999999997E-3</v>
+        <v>7.7220349999999986E-3</v>
       </c>
       <c r="C20">
-        <v>99.623820279787381</v>
+        <v>95.244064290933849</v>
       </c>
       <c r="D20">
-        <v>17.25</v>
+        <v>12.7</v>
       </c>
       <c r="E20">
-        <v>28.95</v>
+        <v>46</v>
       </c>
       <c r="F20">
-        <v>11.6</v>
+        <v>7.7</v>
       </c>
       <c r="G20">
-        <v>29.44648310496456</v>
+        <v>28.558631054322309</v>
       </c>
       <c r="H20">
         <f>_xlfn.VAR.S(B20:F20)</f>
-        <v>1559.5897420428605</v>
+        <v>1545.4379594530731</v>
       </c>
       <c r="I20">
         <f>_xlfn.STDEV.S(B20:F20)</f>
-        <v>39.491641419962029</v>
+        <v>39.312058702808649</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
@@ -1303,385 +1303,385 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B22">
-        <v>7.6949650000000007E-3</v>
+        <v>5.3549600000000006E-3</v>
       </c>
       <c r="C22">
-        <v>96.580674529279761</v>
+        <v>95.466460966906681</v>
       </c>
       <c r="D22">
-        <v>12.7</v>
+        <v>16.75</v>
       </c>
       <c r="E22">
-        <v>46</v>
+        <v>35.049999999999997</v>
       </c>
       <c r="F22">
-        <v>9.1999999999999993</v>
+        <v>9.0500000000000007</v>
       </c>
       <c r="G22">
-        <v>30.414728249046629</v>
+        <v>29.061969321151121</v>
       </c>
       <c r="H22">
         <f>_xlfn.VAR.S(B22:F22)</f>
-        <v>1569.6180029914537</v>
+        <v>1454.3776678210934</v>
       </c>
       <c r="I22">
         <f>_xlfn.STDEV.S(B22:F22)</f>
-        <v>39.618404851677887</v>
+        <v>38.136303803870312</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B23">
-        <v>5.917630000000001E-3</v>
+        <v>5.0783499999999997E-3</v>
       </c>
       <c r="C23">
-        <v>100.0149891043306</v>
+        <v>99.623820279787381</v>
       </c>
       <c r="D23">
-        <v>17.45</v>
+        <v>17.25</v>
       </c>
       <c r="E23">
-        <v>33.4</v>
+        <v>28.95</v>
       </c>
       <c r="F23">
-        <v>10.9</v>
+        <v>11.6</v>
       </c>
       <c r="G23">
-        <v>30.195151122388431</v>
+        <v>29.44648310496456</v>
       </c>
       <c r="H23">
         <f>_xlfn.VAR.S(B23:F23)</f>
-        <v>1576.9763318570535</v>
+        <v>1559.5897420428605</v>
       </c>
       <c r="I23">
         <f>_xlfn.STDEV.S(B23:F23)</f>
-        <v>39.711161300786124</v>
+        <v>39.491641419962029</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="B24">
-        <v>5.7693950000000009E-3</v>
+        <v>4.9714599999999996E-3</v>
       </c>
       <c r="C24">
-        <v>99.450828686644769</v>
+        <v>99.055191129685852</v>
       </c>
       <c r="D24">
-        <v>17</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="E24">
-        <v>31.1</v>
+        <v>30.85</v>
       </c>
       <c r="F24">
-        <v>9.35</v>
+        <v>11.5</v>
       </c>
       <c r="G24">
-        <v>28.05109968027412</v>
+        <v>29.67669376494764</v>
       </c>
       <c r="H24">
         <f>_xlfn.VAR.S(B24:F24)</f>
-        <v>1577.5409388588309</v>
+        <v>1538.6324665253799</v>
       </c>
       <c r="I24">
         <f>_xlfn.STDEV.S(B24:F24)</f>
-        <v>39.71826958540403</v>
+        <v>39.225405880951442</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B25">
-        <v>4.0263149999999999E-3</v>
+        <v>5.0496500000000001E-3</v>
       </c>
       <c r="C25">
-        <v>99.130927060973946</v>
+        <v>102.29869401394031</v>
       </c>
       <c r="D25">
-        <v>11.75</v>
+        <v>15.9</v>
       </c>
       <c r="E25">
-        <v>26.95</v>
+        <v>30.5</v>
       </c>
       <c r="F25">
-        <v>10.85</v>
+        <v>11.3</v>
       </c>
       <c r="G25">
-        <v>27.922492229328981</v>
+        <v>29.892290610656719</v>
       </c>
       <c r="H25">
         <f>_xlfn.VAR.S(B25:F25)</f>
-        <v>1596.8962860240595</v>
+        <v>1663.8833062903916</v>
       </c>
       <c r="I25">
         <f>_xlfn.STDEV.S(B25:F25)</f>
-        <v>39.961184742498055</v>
+        <v>40.790725738706726</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26">
-        <v>4.175425E-3</v>
+        <v>6.2702000000000009E-3</v>
       </c>
       <c r="C26">
-        <v>99.130927060973946</v>
+        <v>95.905800795126837</v>
       </c>
       <c r="D26">
-        <v>11.65</v>
+        <v>15</v>
       </c>
       <c r="E26">
-        <v>27.55</v>
+        <v>41.8</v>
       </c>
       <c r="F26">
-        <v>10.85</v>
+        <v>9.6</v>
       </c>
       <c r="G26">
-        <v>28.005850414328989</v>
+        <v>29.993678499187801</v>
       </c>
       <c r="H26">
         <f>_xlfn.VAR.S(B26:F26)</f>
-        <v>1597.0373141630498</v>
+        <v>1498.3202468311349</v>
       </c>
       <c r="I26">
         <f>_xlfn.STDEV.S(B26:F26)</f>
-        <v>39.962949267578459</v>
+        <v>38.708141867456447</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="B27">
-        <v>4.3338500000000002E-3</v>
+        <v>7.8221300000000001E-3</v>
       </c>
       <c r="C27">
-        <v>99.4652416360247</v>
+        <v>95.466460966906681</v>
       </c>
       <c r="D27">
-        <v>12.45</v>
+        <v>12.25</v>
       </c>
       <c r="E27">
-        <v>27.75</v>
+        <v>46.65</v>
       </c>
       <c r="F27">
-        <v>11.2</v>
+        <v>8.5</v>
       </c>
       <c r="G27">
-        <v>28.378262581004108</v>
+        <v>30.004047182817779</v>
       </c>
       <c r="H27">
         <f>_xlfn.VAR.S(B27:F27)</f>
-        <v>1597.8783877570943</v>
+        <v>1551.6934529663436</v>
       </c>
       <c r="I27">
         <f>_xlfn.STDEV.S(B27:F27)</f>
-        <v>39.973471049648595</v>
+        <v>39.391540373109855</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="B28">
-        <v>4.3084050000000004E-3</v>
+        <v>5.3185200000000002E-3</v>
       </c>
       <c r="C28">
-        <v>99.4652416360247</v>
+        <v>103.8058007951268</v>
       </c>
       <c r="D28">
-        <v>12.45</v>
+        <v>16.95</v>
       </c>
       <c r="E28">
-        <v>27.75</v>
+        <v>32</v>
       </c>
       <c r="F28">
-        <v>11.2</v>
+        <v>9.65</v>
       </c>
       <c r="G28">
-        <v>28.378258340170781</v>
+        <v>30.185186552521131</v>
       </c>
       <c r="H28">
         <f>_xlfn.VAR.S(B28:F28)</f>
-        <v>1597.8787715897215</v>
+        <v>1726.1487428914327</v>
       </c>
       <c r="I28">
         <f>_xlfn.STDEV.S(B28:F28)</f>
-        <v>39.973475850740343</v>
+        <v>41.546946252299129</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B29">
-        <v>5.3969999999999999E-3</v>
+        <v>5.917630000000001E-3</v>
       </c>
       <c r="C29">
-        <v>99.522392368525942</v>
+        <v>100.0149891043306</v>
       </c>
       <c r="D29">
-        <v>16.95</v>
+        <v>17.45</v>
       </c>
       <c r="E29">
-        <v>32</v>
+        <v>33.4</v>
       </c>
       <c r="F29">
-        <v>7.75</v>
+        <v>10.9</v>
       </c>
       <c r="G29">
-        <v>27.662964894754321</v>
+        <v>30.195151122388431</v>
       </c>
       <c r="H29">
         <f>_xlfn.VAR.S(B29:F29)</f>
-        <v>1598.6617944217842</v>
+        <v>1576.9763318570535</v>
       </c>
       <c r="I29">
         <f>_xlfn.STDEV.S(B29:F29)</f>
-        <v>39.983268931163998</v>
+        <v>39.711161300786124</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="B30">
-        <v>6.1662299999999991E-3</v>
+        <v>5.6154550000000001E-3</v>
       </c>
       <c r="C30">
-        <v>101.706662992262</v>
+        <v>103.10960671741429</v>
       </c>
       <c r="D30">
-        <v>17.850000000000001</v>
+        <v>17</v>
       </c>
       <c r="E30">
-        <v>37.700000000000003</v>
+        <v>31.1</v>
       </c>
       <c r="F30">
-        <v>9.6</v>
+        <v>11.65</v>
       </c>
       <c r="G30">
-        <v>30.918804870376999</v>
+        <v>30.352537028735711</v>
       </c>
       <c r="H30">
         <f>_xlfn.VAR.S(B30:F30)</f>
-        <v>1651.9192699580988</v>
+        <v>1679.6268525748019</v>
       </c>
       <c r="I30">
         <f>_xlfn.STDEV.S(B30:F30)</f>
-        <v>40.643809737253946</v>
+        <v>40.983250878557719</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="B31">
-        <v>5.0496500000000001E-3</v>
+        <v>7.6949650000000007E-3</v>
       </c>
       <c r="C31">
-        <v>102.29869401394031</v>
+        <v>96.580674529279761</v>
       </c>
       <c r="D31">
-        <v>15.9</v>
+        <v>12.7</v>
       </c>
       <c r="E31">
-        <v>30.5</v>
+        <v>46</v>
       </c>
       <c r="F31">
-        <v>11.3</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="G31">
-        <v>29.892290610656719</v>
+        <v>30.414728249046629</v>
       </c>
       <c r="H31">
         <f>_xlfn.VAR.S(B31:F31)</f>
-        <v>1663.8833062903916</v>
+        <v>1569.6180029914537</v>
       </c>
       <c r="I31">
         <f>_xlfn.STDEV.S(B31:F31)</f>
-        <v>40.790725738706726</v>
+        <v>39.618404851677887</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="B32">
-        <v>5.6154550000000001E-3</v>
+        <v>6.4687750000000004E-3</v>
       </c>
       <c r="C32">
-        <v>103.10960671741429</v>
+        <v>97.195750288788005</v>
       </c>
       <c r="D32">
-        <v>17</v>
+        <v>14.75</v>
       </c>
       <c r="E32">
-        <v>31.1</v>
+        <v>42.05</v>
       </c>
       <c r="F32">
-        <v>11.65</v>
+        <v>10.25</v>
       </c>
       <c r="G32">
-        <v>30.352537028735711</v>
+        <v>30.483703177298</v>
       </c>
       <c r="H32">
         <f>_xlfn.VAR.S(B32:F32)</f>
-        <v>1679.6268525748019</v>
+        <v>1535.5207806424405</v>
       </c>
       <c r="I32">
         <f>_xlfn.STDEV.S(B32:F32)</f>
-        <v>40.983250878557719</v>
+        <v>39.18572164248657</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="B33">
-        <v>5.3185200000000002E-3</v>
+        <v>6.1662299999999991E-3</v>
       </c>
       <c r="C33">
-        <v>103.8058007951268</v>
+        <v>101.706662992262</v>
       </c>
       <c r="D33">
-        <v>16.95</v>
+        <v>17.850000000000001</v>
       </c>
       <c r="E33">
-        <v>32</v>
+        <v>37.700000000000003</v>
       </c>
       <c r="F33">
-        <v>9.65</v>
+        <v>9.6</v>
       </c>
       <c r="G33">
-        <v>30.185186552521131</v>
+        <v>30.918804870376999</v>
       </c>
       <c r="H33">
         <f>_xlfn.VAR.S(B33:F33)</f>
-        <v>1726.1487428914327</v>
+        <v>1651.9192699580988</v>
       </c>
       <c r="I33">
         <f>_xlfn.STDEV.S(B33:F33)</f>
-        <v>41.546946252299129</v>
+        <v>40.643809737253946</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="B34">
-        <v>9.5076150000000005E-3</v>
+        <v>9.8343599999999986E-3</v>
       </c>
       <c r="C34">
-        <v>99.379812332144624</v>
+        <v>95.051447410283174</v>
       </c>
       <c r="D34">
         <v>242.5</v>
@@ -1690,463 +1690,463 @@
         <v>430.7</v>
       </c>
       <c r="F34">
-        <v>13.7</v>
+        <v>8.5500000000000007</v>
       </c>
       <c r="G34">
-        <v>144.86488665785751</v>
+        <v>131.25188029504719</v>
       </c>
       <c r="H34">
         <f>_xlfn.VAR.S(B34:F34)</f>
-        <v>32680.649564244599</v>
+        <v>33182.366688596609</v>
       </c>
       <c r="I34">
         <f>_xlfn.STDEV.S(B34:F34)</f>
-        <v>180.77790120544213</v>
+        <v>182.160277471782</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B35">
-        <v>9.8343599999999986E-3</v>
+        <v>2.8710469999999998E-2</v>
       </c>
       <c r="C35">
-        <v>95.051447410283174</v>
+        <v>95.942091919212857</v>
       </c>
       <c r="D35">
-        <v>242.5</v>
+        <v>228.45</v>
       </c>
       <c r="E35">
-        <v>430.7</v>
+        <v>456.95</v>
       </c>
       <c r="F35">
-        <v>8.5500000000000007</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="G35">
-        <v>131.25188029504719</v>
+        <v>133.52013373153551</v>
       </c>
       <c r="H35">
         <f>_xlfn.VAR.S(B35:F35)</f>
-        <v>33182.366688596609</v>
+        <v>36350.262859110822</v>
       </c>
       <c r="I35">
         <f>_xlfn.STDEV.S(B35:F35)</f>
-        <v>182.160277471782</v>
+        <v>190.65744899979865</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="B36">
-        <v>2.8290889999999999E-2</v>
+        <v>1.0459725E-2</v>
       </c>
       <c r="C36">
-        <v>101.545140623347</v>
+        <v>96.262525712883303</v>
       </c>
       <c r="D36">
-        <v>228.45</v>
+        <v>231.4</v>
       </c>
       <c r="E36">
-        <v>456.95</v>
+        <v>471.3</v>
       </c>
       <c r="F36">
-        <v>16.7</v>
+        <v>8.4</v>
       </c>
       <c r="G36">
-        <v>148.43723858555779</v>
+        <v>136.3288309063139</v>
       </c>
       <c r="H36">
         <f>_xlfn.VAR.S(B36:F36)</f>
-        <v>35601.203620125525</v>
+        <v>38659.114110763316</v>
       </c>
       <c r="I36">
         <f>_xlfn.STDEV.S(B36:F36)</f>
-        <v>188.68281220112638</v>
+        <v>196.61921094024183</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="B37">
-        <v>2.8710469999999998E-2</v>
+        <v>3.043096E-2</v>
       </c>
       <c r="C37">
-        <v>95.942091919212857</v>
+        <v>97.115190628049064</v>
       </c>
       <c r="D37">
-        <v>228.45</v>
+        <v>229.45</v>
       </c>
       <c r="E37">
-        <v>456.95</v>
+        <v>494</v>
       </c>
       <c r="F37">
-        <v>8.8000000000000007</v>
+        <v>8.6</v>
       </c>
       <c r="G37">
-        <v>133.52013373153551</v>
+        <v>139.98260359800821</v>
       </c>
       <c r="H37">
         <f>_xlfn.VAR.S(B37:F37)</f>
-        <v>36350.262859110822</v>
+        <v>42168.886976151858</v>
       </c>
       <c r="I37">
         <f>_xlfn.STDEV.S(B37:F37)</f>
-        <v>190.65744899979865</v>
+        <v>205.35064396332402</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="B38">
-        <v>1.011546E-2</v>
+        <v>1.5185805E-2</v>
       </c>
       <c r="C38">
-        <v>100.3383909759073</v>
+        <v>96.304366757830977</v>
       </c>
       <c r="D38">
-        <v>231.4</v>
+        <v>217.9</v>
       </c>
       <c r="E38">
-        <v>471.3</v>
+        <v>528.20000000000005</v>
       </c>
       <c r="F38">
-        <v>13.4</v>
+        <v>9.15</v>
       </c>
       <c r="G38">
-        <v>150.05808440598449</v>
+        <v>143.79492542713851</v>
       </c>
       <c r="H38">
         <f>_xlfn.VAR.S(B38:F38)</f>
-        <v>38149.842518417965</v>
+        <v>47699.940804205857</v>
       </c>
       <c r="I38">
         <f>_xlfn.STDEV.S(B38:F38)</f>
-        <v>195.3198467089762</v>
+        <v>218.40316115891238</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>49</v>
+        <v>14</v>
       </c>
       <c r="B39">
-        <v>1.0459725E-2</v>
+        <v>9.5076150000000005E-3</v>
       </c>
       <c r="C39">
-        <v>96.262525712883303</v>
+        <v>99.379812332144624</v>
       </c>
       <c r="D39">
-        <v>231.4</v>
+        <v>242.5</v>
       </c>
       <c r="E39">
-        <v>471.3</v>
+        <v>430.7</v>
       </c>
       <c r="F39">
-        <v>8.4</v>
+        <v>13.7</v>
       </c>
       <c r="G39">
-        <v>136.3288309063139</v>
+        <v>144.86488665785751</v>
       </c>
       <c r="H39">
         <f>_xlfn.VAR.S(B39:F39)</f>
-        <v>38659.114110763316</v>
+        <v>32680.649564244599</v>
       </c>
       <c r="I39">
         <f>_xlfn.STDEV.S(B39:F39)</f>
-        <v>196.61921094024183</v>
+        <v>180.77790120544213</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="B40">
-        <v>3.0107795E-2</v>
+        <v>1.439782E-2</v>
       </c>
       <c r="C40">
-        <v>102.72798333582161</v>
+        <v>96.11554805056582</v>
       </c>
       <c r="D40">
-        <v>229.45</v>
+        <v>232.5</v>
       </c>
       <c r="E40">
-        <v>494</v>
+        <v>522.54999999999995</v>
       </c>
       <c r="F40">
-        <v>14.35</v>
+        <v>9.1</v>
       </c>
       <c r="G40">
-        <v>154.76801518847029</v>
+        <v>145.2466576450943</v>
       </c>
       <c r="H40">
         <f>_xlfn.VAR.S(B40:F40)</f>
-        <v>41533.670888406501</v>
+        <v>47104.861057736271</v>
       </c>
       <c r="I40">
         <f>_xlfn.STDEV.S(B40:F40)</f>
-        <v>203.79811306390081</v>
+        <v>217.03654313902135</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="B41">
-        <v>3.043096E-2</v>
+        <v>3.4688625000000001E-2</v>
       </c>
       <c r="C41">
-        <v>97.115190628049064</v>
+        <v>96.343053687454997</v>
       </c>
       <c r="D41">
-        <v>229.45</v>
+        <v>223.4</v>
       </c>
       <c r="E41">
-        <v>494</v>
+        <v>536.6</v>
       </c>
       <c r="F41">
-        <v>8.6</v>
+        <v>9.1</v>
       </c>
       <c r="G41">
-        <v>139.98260359800821</v>
+        <v>146.10462371874249</v>
       </c>
       <c r="H41">
         <f>_xlfn.VAR.S(B41:F41)</f>
-        <v>42168.886976151858</v>
+        <v>49350.39267736792</v>
       </c>
       <c r="I41">
         <f>_xlfn.STDEV.S(B41:F41)</f>
-        <v>205.35064396332402</v>
+        <v>222.14948273036316</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="B42">
-        <v>1.402522E-2</v>
+        <v>3.5856364999999987E-2</v>
       </c>
       <c r="C42">
-        <v>100.0865619795843</v>
+        <v>96.470693022813506</v>
       </c>
       <c r="D42">
-        <v>232.5</v>
+        <v>222.45</v>
       </c>
       <c r="E42">
-        <v>522.54999999999995</v>
+        <v>543.5</v>
       </c>
       <c r="F42">
-        <v>13.95</v>
+        <v>9.35</v>
       </c>
       <c r="G42">
-        <v>159.09176453326401</v>
+        <v>147.19275823130221</v>
       </c>
       <c r="H42">
         <f>_xlfn.VAR.S(B42:F42)</f>
-        <v>46564.877237866858</v>
+        <v>50565.234746720889</v>
       </c>
       <c r="I42">
         <f>_xlfn.STDEV.S(B42:F42)</f>
-        <v>215.78896458778161</v>
+        <v>224.86714910524589</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>64</v>
+        <v>9</v>
       </c>
       <c r="B43">
-        <v>1.439782E-2</v>
+        <v>2.8290889999999999E-2</v>
       </c>
       <c r="C43">
-        <v>96.11554805056582</v>
+        <v>101.545140623347</v>
       </c>
       <c r="D43">
-        <v>232.5</v>
+        <v>228.45</v>
       </c>
       <c r="E43">
-        <v>522.54999999999995</v>
+        <v>456.95</v>
       </c>
       <c r="F43">
-        <v>9.1</v>
+        <v>16.7</v>
       </c>
       <c r="G43">
-        <v>145.2466576450943</v>
+        <v>148.43723858555779</v>
       </c>
       <c r="H43">
         <f>_xlfn.VAR.S(B43:F43)</f>
-        <v>47104.861057736271</v>
+        <v>35601.203620125525</v>
       </c>
       <c r="I43">
         <f>_xlfn.STDEV.S(B43:F43)</f>
-        <v>217.03654313902135</v>
+        <v>188.68281220112638</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B44">
-        <v>1.482062E-2</v>
+        <v>1.011546E-2</v>
       </c>
       <c r="C44">
-        <v>100.5259018078045</v>
+        <v>100.3383909759073</v>
       </c>
       <c r="D44">
-        <v>217.9</v>
+        <v>231.4</v>
       </c>
       <c r="E44">
-        <v>528.20000000000005</v>
+        <v>471.3</v>
       </c>
       <c r="F44">
-        <v>14.4</v>
+        <v>13.4</v>
       </c>
       <c r="G44">
-        <v>157.8734537379674</v>
+        <v>150.05808440598449</v>
       </c>
       <c r="H44">
         <f>_xlfn.VAR.S(B44:F44)</f>
-        <v>47127.560504531015</v>
+        <v>38149.842518417965</v>
       </c>
       <c r="I44">
         <f>_xlfn.STDEV.S(B44:F44)</f>
-        <v>217.08883090691472</v>
+        <v>195.3198467089762</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="B45">
-        <v>1.5185805E-2</v>
+        <v>3.0107795E-2</v>
       </c>
       <c r="C45">
-        <v>96.304366757830977</v>
+        <v>102.72798333582161</v>
       </c>
       <c r="D45">
-        <v>217.9</v>
+        <v>229.45</v>
       </c>
       <c r="E45">
-        <v>528.20000000000005</v>
+        <v>494</v>
       </c>
       <c r="F45">
-        <v>9.15</v>
+        <v>14.35</v>
       </c>
       <c r="G45">
-        <v>143.79492542713851</v>
+        <v>154.76801518847029</v>
       </c>
       <c r="H45">
         <f>_xlfn.VAR.S(B45:F45)</f>
-        <v>47699.940804205857</v>
+        <v>41533.670888406501</v>
       </c>
       <c r="I45">
         <f>_xlfn.STDEV.S(B45:F45)</f>
-        <v>218.40316115891238</v>
+        <v>203.79811306390081</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B46">
-        <v>3.433538500000001E-2</v>
+        <v>1.482062E-2</v>
       </c>
       <c r="C46">
-        <v>100.706662992262</v>
+        <v>100.5259018078045</v>
       </c>
       <c r="D46">
-        <v>223.4</v>
+        <v>217.9</v>
       </c>
       <c r="E46">
-        <v>536.6</v>
+        <v>528.20000000000005</v>
       </c>
       <c r="F46">
-        <v>13.9</v>
+        <v>14.4</v>
       </c>
       <c r="G46">
-        <v>160.21516639621029</v>
+        <v>157.8734537379674</v>
       </c>
       <c r="H46">
         <f>_xlfn.VAR.S(B46:F46)</f>
-        <v>48795.696985370254</v>
+        <v>47127.560504531015</v>
       </c>
       <c r="I46">
         <f>_xlfn.STDEV.S(B46:F46)</f>
-        <v>220.89748071304538</v>
+        <v>217.08883090691472</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B47">
-        <v>3.4688625000000001E-2</v>
+        <v>1.402522E-2</v>
       </c>
       <c r="C47">
-        <v>96.343053687454997</v>
+        <v>100.0865619795843</v>
       </c>
       <c r="D47">
-        <v>223.4</v>
+        <v>232.5</v>
       </c>
       <c r="E47">
-        <v>536.6</v>
+        <v>522.54999999999995</v>
       </c>
       <c r="F47">
-        <v>9.1</v>
+        <v>13.95</v>
       </c>
       <c r="G47">
-        <v>146.10462371874249</v>
+        <v>159.09176453326401</v>
       </c>
       <c r="H47">
         <f>_xlfn.VAR.S(B47:F47)</f>
-        <v>49350.39267736792</v>
+        <v>46564.877237866858</v>
       </c>
       <c r="I47">
         <f>_xlfn.STDEV.S(B47:F47)</f>
-        <v>222.14948273036316</v>
+        <v>215.78896458778161</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="B48">
-        <v>3.5589095000000001E-2</v>
+        <v>3.433538500000001E-2</v>
       </c>
       <c r="C48">
-        <v>101.5259018078045</v>
+        <v>100.706662992262</v>
       </c>
       <c r="D48">
-        <v>222.45</v>
+        <v>223.4</v>
       </c>
       <c r="E48">
-        <v>543.5</v>
+        <v>536.6</v>
       </c>
       <c r="F48">
-        <v>14.65</v>
+        <v>13.9</v>
       </c>
       <c r="G48">
-        <v>161.56024848380071</v>
+        <v>160.21516639621029</v>
       </c>
       <c r="H48">
         <f>_xlfn.VAR.S(B48:F48)</f>
-        <v>49939.151449524965</v>
+        <v>48795.696985370254</v>
       </c>
       <c r="I48">
         <f>_xlfn.STDEV.S(B48:F48)</f>
-        <v>223.4706948338528</v>
+        <v>220.89748071304538</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="B49">
-        <v>3.5856364999999987E-2</v>
+        <v>3.5589095000000001E-2</v>
       </c>
       <c r="C49">
-        <v>96.470693022813506</v>
+        <v>101.5259018078045</v>
       </c>
       <c r="D49">
         <v>222.45</v>
@@ -2155,29 +2155,29 @@
         <v>543.5</v>
       </c>
       <c r="F49">
-        <v>9.35</v>
+        <v>14.65</v>
       </c>
       <c r="G49">
-        <v>147.19275823130221</v>
+        <v>161.56024848380071</v>
       </c>
       <c r="H49">
         <f>_xlfn.VAR.S(B49:F49)</f>
-        <v>50565.234746720889</v>
+        <v>49939.151449524965</v>
       </c>
       <c r="I49">
         <f>_xlfn.STDEV.S(B49:F49)</f>
-        <v>224.86714910524589</v>
+        <v>223.4706948338528</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="B50">
-        <v>8.0202699999999995E-3</v>
+        <v>8.3724000000000003E-3</v>
       </c>
       <c r="C50">
-        <v>99.415851301465665</v>
+        <v>94.96604375813385</v>
       </c>
       <c r="D50">
         <v>207.35</v>
@@ -2186,91 +2186,91 @@
         <v>890.75</v>
       </c>
       <c r="F50">
-        <v>15.95</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="G50">
-        <v>216.37897859524429</v>
+        <v>202.33740269302231</v>
       </c>
       <c r="H50">
         <f>_xlfn.VAR.S(B50:F50)</f>
-        <v>138015.93291424785</v>
+        <v>139098.44430271158</v>
       </c>
       <c r="I50">
         <f>_xlfn.STDEV.S(B50:F50)</f>
-        <v>371.50495678287774</v>
+        <v>372.95903837112138</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="B51">
-        <v>8.3724000000000003E-3</v>
+        <v>8.5663300000000005E-3</v>
       </c>
       <c r="C51">
-        <v>94.96604375813385</v>
+        <v>94.983149630726132</v>
       </c>
       <c r="D51">
-        <v>207.35</v>
+        <v>214.7</v>
       </c>
       <c r="E51">
-        <v>890.75</v>
+        <v>903.35</v>
       </c>
       <c r="F51">
-        <v>9.3000000000000007</v>
+        <v>9.25</v>
       </c>
       <c r="G51">
-        <v>202.33740269302231</v>
+        <v>205.64028599345431</v>
       </c>
       <c r="H51">
         <f>_xlfn.VAR.S(B51:F51)</f>
-        <v>139098.44430271158</v>
+        <v>143111.31650147791</v>
       </c>
       <c r="I51">
         <f>_xlfn.STDEV.S(B51:F51)</f>
-        <v>372.95903837112138</v>
+        <v>378.30056370758678</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="B52">
-        <v>8.2059100000000003E-3</v>
+        <v>8.0202699999999995E-3</v>
       </c>
       <c r="C52">
-        <v>99.652247404533583</v>
+        <v>99.415851301465665</v>
       </c>
       <c r="D52">
-        <v>214.7</v>
+        <v>207.35</v>
       </c>
       <c r="E52">
-        <v>903.35</v>
+        <v>890.75</v>
       </c>
       <c r="F52">
-        <v>16</v>
+        <v>15.95</v>
       </c>
       <c r="G52">
-        <v>219.76007555242231</v>
+        <v>216.37897859524429</v>
       </c>
       <c r="H52">
         <f>_xlfn.VAR.S(B52:F52)</f>
-        <v>141978.89661415026</v>
+        <v>138015.93291424785</v>
       </c>
       <c r="I52">
         <f>_xlfn.STDEV.S(B52:F52)</f>
-        <v>376.80087130227054</v>
+        <v>371.50495678287774</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="B53">
-        <v>8.5663300000000005E-3</v>
+        <v>8.2059100000000003E-3</v>
       </c>
       <c r="C53">
-        <v>94.983149630726132</v>
+        <v>99.652247404533583</v>
       </c>
       <c r="D53">
         <v>214.7</v>
@@ -2279,29 +2279,29 @@
         <v>903.35</v>
       </c>
       <c r="F53">
-        <v>9.25</v>
+        <v>16</v>
       </c>
       <c r="G53">
-        <v>205.64028599345431</v>
+        <v>219.76007555242231</v>
       </c>
       <c r="H53">
         <f>_xlfn.VAR.S(B53:F53)</f>
-        <v>143111.31650147791</v>
+        <v>141978.89661415026</v>
       </c>
       <c r="I53">
         <f>_xlfn.STDEV.S(B53:F53)</f>
-        <v>378.30056370758678</v>
+        <v>376.80087130227054</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="B54">
-        <v>3.9248825000000001E-2</v>
+        <v>3.9593120000000002E-2</v>
       </c>
       <c r="C54">
-        <v>95.8765114732455</v>
+        <v>91.984921200877267</v>
       </c>
       <c r="D54">
         <v>221.85</v>
@@ -2310,215 +2310,215 @@
         <v>1060.95</v>
       </c>
       <c r="F54">
-        <v>11.7</v>
+        <v>7.9</v>
       </c>
       <c r="G54">
-        <v>245.22762671637429</v>
+        <v>232.1040857201462</v>
       </c>
       <c r="H54">
         <f>_xlfn.VAR.S(B54:F54)</f>
-        <v>199377.58117389996</v>
+        <v>200242.63644879134</v>
       </c>
       <c r="I54">
         <f>_xlfn.STDEV.S(B54:F54)</f>
-        <v>446.51716783781109</v>
+        <v>447.48478906974185</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="B55">
-        <v>3.9593120000000002E-2</v>
+        <v>3.7452159999999998E-2</v>
       </c>
       <c r="C55">
-        <v>91.984921200877267</v>
+        <v>92.095917778269126</v>
       </c>
       <c r="D55">
-        <v>221.85</v>
+        <v>244.05</v>
       </c>
       <c r="E55">
-        <v>1060.95</v>
+        <v>1071</v>
       </c>
       <c r="F55">
-        <v>7.9</v>
+        <v>7.85</v>
       </c>
       <c r="G55">
-        <v>232.1040857201462</v>
+        <v>237.4888949897115</v>
       </c>
       <c r="H55">
         <f>_xlfn.VAR.S(B55:F55)</f>
-        <v>200242.63644879134</v>
+        <v>203670.19921657883</v>
       </c>
       <c r="I55">
         <f>_xlfn.STDEV.S(B55:F55)</f>
-        <v>447.48478906974185</v>
+        <v>451.29834834240069</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="B56">
-        <v>3.7197380000000002E-2</v>
+        <v>7.5084250000000009E-3</v>
       </c>
       <c r="C56">
-        <v>95.993668760770873</v>
+        <v>92.206496440983841</v>
       </c>
       <c r="D56">
-        <v>244.05</v>
+        <v>257.25</v>
       </c>
       <c r="E56">
-        <v>1071</v>
+        <v>1094.5</v>
       </c>
       <c r="F56">
-        <v>11.7</v>
+        <v>7</v>
       </c>
       <c r="G56">
-        <v>250.6551443567952</v>
+        <v>243.335667477664</v>
       </c>
       <c r="H56">
         <f>_xlfn.VAR.S(B56:F56)</f>
-        <v>202772.99992863525</v>
+        <v>212899.88546473763</v>
       </c>
       <c r="I56">
         <f>_xlfn.STDEV.S(B56:F56)</f>
-        <v>450.3032310883803</v>
+        <v>461.4107556881803</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="B57">
-        <v>3.7452159999999998E-2</v>
+        <v>3.9248825000000001E-2</v>
       </c>
       <c r="C57">
-        <v>92.095917778269126</v>
+        <v>95.8765114732455</v>
       </c>
       <c r="D57">
-        <v>244.05</v>
+        <v>221.85</v>
       </c>
       <c r="E57">
-        <v>1071</v>
+        <v>1060.95</v>
       </c>
       <c r="F57">
-        <v>7.85</v>
+        <v>11.7</v>
       </c>
       <c r="G57">
-        <v>237.4888949897115</v>
+        <v>245.22762671637429</v>
       </c>
       <c r="H57">
         <f>_xlfn.VAR.S(B57:F57)</f>
-        <v>203670.19921657883</v>
+        <v>199377.58117389996</v>
       </c>
       <c r="I57">
         <f>_xlfn.STDEV.S(B57:F57)</f>
-        <v>451.29834834240069</v>
+        <v>446.51716783781109</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B58">
-        <v>7.1566900000000003E-3</v>
+        <v>3.7197380000000002E-2</v>
       </c>
       <c r="C58">
-        <v>95.992806563635739</v>
+        <v>95.993668760770873</v>
       </c>
       <c r="D58">
-        <v>257.25</v>
+        <v>244.05</v>
       </c>
       <c r="E58">
-        <v>1094.5</v>
+        <v>1071</v>
       </c>
       <c r="F58">
-        <v>12.05</v>
+        <v>11.7</v>
       </c>
       <c r="G58">
-        <v>256.68332720893932</v>
+        <v>250.6551443567952</v>
       </c>
       <c r="H58">
         <f>_xlfn.VAR.S(B58:F58)</f>
-        <v>211816.11185502959</v>
+        <v>202772.99992863525</v>
       </c>
       <c r="I58">
         <f>_xlfn.STDEV.S(B58:F58)</f>
-        <v>460.23484424262097</v>
+        <v>450.3032310883803</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="B59">
-        <v>7.5084250000000009E-3</v>
+        <v>7.1844350000000003E-3</v>
       </c>
       <c r="C59">
-        <v>92.206496440983841</v>
+        <v>91.985986402328749</v>
       </c>
       <c r="D59">
-        <v>257.25</v>
+        <v>304.85000000000002</v>
       </c>
       <c r="E59">
-        <v>1094.5</v>
+        <v>1118.4000000000001</v>
       </c>
       <c r="F59">
-        <v>7</v>
+        <v>7.15</v>
       </c>
       <c r="G59">
-        <v>243.335667477664</v>
+        <v>255.2821951395548</v>
       </c>
       <c r="H59">
         <f>_xlfn.VAR.S(B59:F59)</f>
-        <v>212899.88546473763</v>
+        <v>222182.10835589963</v>
       </c>
       <c r="I59">
         <f>_xlfn.STDEV.S(B59:F59)</f>
-        <v>461.4107556881803</v>
+        <v>471.3619716904405</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B60">
-        <v>6.821405E-3</v>
+        <v>7.1566900000000003E-3</v>
       </c>
       <c r="C60">
-        <v>96.046359954229004</v>
+        <v>95.992806563635739</v>
       </c>
       <c r="D60">
-        <v>304.85000000000002</v>
+        <v>257.25</v>
       </c>
       <c r="E60">
-        <v>1118.4000000000001</v>
+        <v>1094.5</v>
       </c>
       <c r="F60">
-        <v>12.6</v>
+        <v>12.05</v>
       </c>
       <c r="G60">
-        <v>268.69219689320488</v>
+        <v>256.68332720893932</v>
       </c>
       <c r="H60">
         <f>_xlfn.VAR.S(B60:F60)</f>
-        <v>220947.56859882094</v>
+        <v>211816.11185502959</v>
       </c>
       <c r="I60">
         <f>_xlfn.STDEV.S(B60:F60)</f>
-        <v>470.05060216834204</v>
+        <v>460.23484424262097</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B61">
-        <v>7.1844350000000003E-3</v>
+        <v>6.821405E-3</v>
       </c>
       <c r="C61">
-        <v>91.985986402328749</v>
+        <v>96.046359954229004</v>
       </c>
       <c r="D61">
         <v>304.85000000000002</v>
@@ -2527,29 +2527,29 @@
         <v>1118.4000000000001</v>
       </c>
       <c r="F61">
-        <v>7.15</v>
+        <v>12.6</v>
       </c>
       <c r="G61">
-        <v>255.2821951395548</v>
+        <v>268.69219689320488</v>
       </c>
       <c r="H61">
         <f>_xlfn.VAR.S(B61:F61)</f>
-        <v>222182.10835589963</v>
+        <v>220947.56859882094</v>
       </c>
       <c r="I61">
         <f>_xlfn.STDEV.S(B61:F61)</f>
-        <v>471.3619716904405</v>
+        <v>470.05060216834204</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B62">
-        <v>5.8780910000000013E-2</v>
+        <v>5.8907709999999988E-2</v>
       </c>
       <c r="C62">
-        <v>95.466460966906681</v>
+        <v>92.482902311963187</v>
       </c>
       <c r="D62">
         <v>265.10000000000002</v>
@@ -2558,91 +2558,91 @@
         <v>1574.9</v>
       </c>
       <c r="F62">
-        <v>19.8</v>
+        <v>6.75</v>
       </c>
       <c r="G62">
-        <v>339.2625403128178</v>
+        <v>324.67363500366048</v>
       </c>
       <c r="H62">
         <f>_xlfn.VAR.S(B62:F62)</f>
-        <v>448858.63708013622</v>
+        <v>451754.03207662748</v>
       </c>
       <c r="I62">
         <f>_xlfn.STDEV.S(B62:F62)</f>
-        <v>669.96913143825975</v>
+        <v>672.12650005532998</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B63">
-        <v>5.8907709999999988E-2</v>
+        <v>5.7396324999999991E-2</v>
       </c>
       <c r="C63">
-        <v>92.482902311963187</v>
+        <v>92.33396854170924</v>
       </c>
       <c r="D63">
-        <v>265.10000000000002</v>
+        <v>235.5</v>
       </c>
       <c r="E63">
-        <v>1574.9</v>
+        <v>1610.25</v>
       </c>
       <c r="F63">
         <v>6.75</v>
       </c>
       <c r="G63">
-        <v>324.67363500366048</v>
+        <v>325.61522747778491</v>
       </c>
       <c r="H63">
         <f>_xlfn.VAR.S(B63:F63)</f>
-        <v>451754.03207662748</v>
+        <v>475103.98895359534</v>
       </c>
       <c r="I63">
         <f>_xlfn.STDEV.S(B63:F63)</f>
-        <v>672.12650005532998</v>
+        <v>689.27787499207841</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B64">
-        <v>5.7199159999999992E-2</v>
+        <v>5.8780910000000013E-2</v>
       </c>
       <c r="C64">
         <v>95.466460966906681</v>
       </c>
       <c r="D64">
-        <v>235.5</v>
+        <v>265.10000000000002</v>
       </c>
       <c r="E64">
-        <v>1610.25</v>
+        <v>1574.9</v>
       </c>
       <c r="F64">
-        <v>14.4</v>
+        <v>19.8</v>
       </c>
       <c r="G64">
-        <v>339.32061002115108</v>
+        <v>339.2625403128178</v>
       </c>
       <c r="H64">
         <f>_xlfn.VAR.S(B64:F64)</f>
-        <v>473188.65698961378</v>
+        <v>448858.63708013622</v>
       </c>
       <c r="I64">
         <f>_xlfn.STDEV.S(B64:F64)</f>
-        <v>687.88709610634055</v>
+        <v>669.96913143825975</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="B65">
-        <v>5.7396324999999991E-2</v>
+        <v>5.7199159999999992E-2</v>
       </c>
       <c r="C65">
-        <v>92.33396854170924</v>
+        <v>95.466460966906681</v>
       </c>
       <c r="D65">
         <v>235.5</v>
@@ -2651,24 +2651,24 @@
         <v>1610.25</v>
       </c>
       <c r="F65">
-        <v>6.75</v>
+        <v>14.4</v>
       </c>
       <c r="G65">
-        <v>325.61522747778491</v>
+        <v>339.32061002115108</v>
       </c>
       <c r="H65">
         <f>_xlfn.VAR.S(B65:F65)</f>
-        <v>475103.98895359534</v>
+        <v>473188.65698961378</v>
       </c>
       <c r="I65">
         <f>_xlfn.STDEV.S(B65:F65)</f>
-        <v>689.27787499207841</v>
+        <v>687.88709610634055</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I65" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I65">
-      <sortCondition ref="I1:I65"/>
+      <sortCondition ref="G1:G65"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
checkout sebelum perubahan Path Polyline Optimization
</commit_message>
<xml_diff>
--- a/Excel/Rekap/Avg_Keseluruhan_All.xlsx
+++ b/Excel/Rekap/Avg_Keseluruhan_All.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEMHAS\TA_Python_Server\Excel\Rekap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A4CF30-F0B4-48B1-9E29-B12D8FC383BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57EFA7B8-421D-428C-B58A-D04C9831B616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,23 +18,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$49</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>Kombinasi</t>
   </si>
@@ -202,16 +191,13 @@
   </si>
   <si>
     <t>JPS-BDS-GL-BRC-PPO</t>
-  </si>
-  <si>
-    <t>total</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -227,14 +213,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -249,18 +229,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -283,32 +257,17 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -613,7 +572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" bestFit="1" customWidth="1"/>
@@ -623,10 +582,9 @@
     <col min="5" max="5" width="16.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -651,21 +609,18 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>42</v>
       </c>
       <c r="B2">
-        <v>3.5538050000000002E-3</v>
+        <v>3.5719649999999999E-3</v>
       </c>
       <c r="C2">
         <v>10.6</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="3">
         <v>96.016010671277556</v>
       </c>
       <c r="E2">
@@ -678,20 +633,15 @@
         <v>8.6</v>
       </c>
       <c r="H2">
-        <f>AVERAGE(B2:D2,I2,G2)</f>
-        <v>30.123912895255511</v>
-      </c>
-      <c r="I2">
-        <f>SUM(E2:F2)</f>
-        <v>35.4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+        <v>25.103263772712921</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>53</v>
       </c>
       <c r="B3">
-        <v>3.8192349999999998E-3</v>
+        <v>3.8451199999999992E-3</v>
       </c>
       <c r="C3">
         <v>10.6</v>
@@ -709,20 +659,15 @@
         <v>8.6</v>
       </c>
       <c r="H3">
-        <f>AVERAGE(B3:D3,I3,G3)</f>
-        <v>30.475979217092011</v>
-      </c>
-      <c r="I3">
-        <f t="shared" ref="I3:I49" si="0">SUM(E3:F3)</f>
-        <v>37.700000000000003</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+        <v>25.39665366174334</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>41</v>
       </c>
       <c r="B4">
-        <v>5.1365749999999991E-3</v>
+        <v>5.1926349999999993E-3</v>
       </c>
       <c r="C4">
         <v>9.6</v>
@@ -740,51 +685,41 @@
         <v>7.6</v>
       </c>
       <c r="H4">
-        <f>AVERAGE(B4:D4,I4,G4)</f>
-        <v>31.801737556421649</v>
-      </c>
-      <c r="I4">
-        <f t="shared" si="0"/>
-        <v>49.65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+        <v>26.50145730701804</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="4">
-        <v>5.0321199999999993E-3</v>
-      </c>
-      <c r="C5" s="4">
+      <c r="B5" s="2">
+        <v>5.1205399999999998E-3</v>
+      </c>
+      <c r="C5" s="2">
         <v>10.65</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="2">
         <v>94.328115771513964</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="2">
         <v>16.7</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="2">
         <v>29.65</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="2">
         <v>8.6</v>
       </c>
-      <c r="H5" s="4">
-        <f>AVERAGE(B5:D5,I5,G5)</f>
-        <v>31.986629578302789</v>
-      </c>
-      <c r="I5" s="4">
-        <f t="shared" si="0"/>
-        <v>46.349999999999994</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H5" s="2">
+        <v>26.655539385252329</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>25</v>
       </c>
       <c r="B6">
-        <v>3.4819349999999998E-3</v>
+        <v>3.52353E-3</v>
       </c>
       <c r="C6">
         <v>18.8</v>
@@ -802,20 +737,15 @@
         <v>10.45</v>
       </c>
       <c r="H6">
-        <f>AVERAGE(B6:D6,I6,G6)</f>
-        <v>32.484749764838817</v>
-      </c>
-      <c r="I6">
-        <f t="shared" si="0"/>
-        <v>35.4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+        <v>27.070631736532349</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>44</v>
       </c>
       <c r="B7">
-        <v>5.5173499999999999E-3</v>
+        <v>5.5573150000000002E-3</v>
       </c>
       <c r="C7">
         <v>9.75</v>
@@ -833,20 +763,15 @@
         <v>7.75</v>
       </c>
       <c r="H7">
-        <f>AVERAGE(B7:D7,I7,G7)</f>
-        <v>32.848227342779836</v>
-      </c>
-      <c r="I7">
-        <f t="shared" si="0"/>
-        <v>53.7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+        <v>27.37352944648319</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
       <c r="B8">
-        <v>3.7062649999999998E-3</v>
+        <v>3.77189E-3</v>
       </c>
       <c r="C8">
         <v>19.05</v>
@@ -864,51 +789,41 @@
         <v>10.4</v>
       </c>
       <c r="H8">
-        <f>AVERAGE(B8:D8,I8,G8)</f>
-        <v>32.902784529571058</v>
-      </c>
-      <c r="I8">
-        <f t="shared" si="0"/>
-        <v>37.700000000000003</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+        <v>27.418998045475881</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B9" s="3">
-        <v>5.347494999999999E-3</v>
-      </c>
-      <c r="C9" s="3">
+      <c r="B9" s="2">
+        <v>5.4922499999999997E-3</v>
+      </c>
+      <c r="C9" s="2">
         <v>10.75</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <v>94.585481455216581</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="2">
         <v>18.95</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="2">
         <v>31.6</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="2">
         <v>8.6999999999999993</v>
       </c>
-      <c r="H9" s="3">
-        <f>AVERAGE(B9:D9,I9,G9)</f>
-        <v>32.918165790043318</v>
-      </c>
-      <c r="I9" s="3">
-        <f t="shared" si="0"/>
-        <v>50.55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H9" s="2">
+        <v>27.431828950869431</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>27</v>
       </c>
       <c r="B10">
-        <v>6.58598E-3</v>
+        <v>6.6073800000000004E-3</v>
       </c>
       <c r="C10">
         <v>9.6</v>
@@ -926,20 +841,15 @@
         <v>7.6</v>
       </c>
       <c r="H10">
-        <f>AVERAGE(B10:D10,I10,G10)</f>
-        <v>33.364995085886072</v>
-      </c>
-      <c r="I10">
-        <f t="shared" si="0"/>
-        <v>56.1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+        <v>27.804166138238401</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>52</v>
       </c>
       <c r="B11">
-        <v>5.7534149999999996E-3</v>
+        <v>5.8775849999999994E-3</v>
       </c>
       <c r="C11">
         <v>10.65</v>
@@ -957,20 +867,15 @@
         <v>8.5500000000000007</v>
       </c>
       <c r="H11">
-        <f>AVERAGE(B11:D11,I11,G11)</f>
-        <v>33.796123154933689</v>
-      </c>
-      <c r="I11">
-        <f t="shared" si="0"/>
-        <v>55.599999999999994</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+        <v>28.16345665744474</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>24</v>
       </c>
       <c r="B12">
-        <v>5.0736500000000007E-3</v>
+        <v>5.14387E-3</v>
       </c>
       <c r="C12">
         <v>18.8</v>
@@ -988,20 +893,15 @@
         <v>9.4</v>
       </c>
       <c r="H12">
-        <f>AVERAGE(B12:D12,I12,G12)</f>
-        <v>34.488570992093265</v>
-      </c>
-      <c r="I12">
-        <f t="shared" si="0"/>
-        <v>49.65</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+        <v>28.740487530077719</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>39</v>
       </c>
       <c r="B13">
-        <v>4.9429149999999991E-3</v>
+        <v>5.0282450000000006E-3</v>
       </c>
       <c r="C13">
         <v>18.8</v>
@@ -1019,20 +919,15 @@
         <v>10.6</v>
       </c>
       <c r="H13">
-        <f>AVERAGE(B13:D13,I13,G13)</f>
-        <v>34.568889723947322</v>
-      </c>
-      <c r="I13">
-        <f t="shared" si="0"/>
-        <v>46.349999999999994</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+        <v>28.8074223249561</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>26</v>
       </c>
       <c r="B14">
-        <v>5.40779E-3</v>
+        <v>5.4405850000000004E-3</v>
       </c>
       <c r="C14">
         <v>18.3</v>
@@ -1050,51 +945,41 @@
         <v>9.4</v>
       </c>
       <c r="H14">
-        <f>AVERAGE(B14:D14,I14,G14)</f>
-        <v>35.204495684469535</v>
-      </c>
-      <c r="I14">
-        <f t="shared" si="0"/>
-        <v>53.7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+        <v>29.33708520289127</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B15">
-        <v>6.516875000000001E-3</v>
-      </c>
-      <c r="C15">
+      <c r="B15" s="2">
+        <v>6.587599999999999E-3</v>
+      </c>
+      <c r="C15" s="2">
         <v>18.149999999999999</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="2">
         <v>94.587781310466312</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="2">
         <v>13.1</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="2">
         <v>43</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="2">
         <v>8.9</v>
       </c>
-      <c r="H15">
-        <f>AVERAGE(B15:D15,I15,G15)</f>
-        <v>35.548859637093258</v>
-      </c>
-      <c r="I15">
-        <f t="shared" si="0"/>
-        <v>56.1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H15" s="2">
+        <v>29.624061485077721</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>51</v>
       </c>
       <c r="B16">
-        <v>5.2956100000000001E-3</v>
+        <v>5.4088249999999999E-3</v>
       </c>
       <c r="C16">
         <v>19.350000000000001</v>
@@ -1112,20 +997,15 @@
         <v>11.15</v>
       </c>
       <c r="H16">
-        <f>AVERAGE(B16:D16,I16,G16)</f>
-        <v>35.714818127323596</v>
-      </c>
-      <c r="I16">
-        <f t="shared" si="0"/>
-        <v>50.55</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+        <v>29.76236730860299</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>40</v>
       </c>
       <c r="B17">
-        <v>5.6697400000000012E-3</v>
+        <v>5.7431750000000014E-3</v>
       </c>
       <c r="C17">
         <v>19.350000000000001</v>
@@ -1143,20 +1023,15 @@
         <v>11.05</v>
       </c>
       <c r="H17">
-        <f>AVERAGE(B17:D17,I17,G17)</f>
-        <v>36.591167123303286</v>
-      </c>
-      <c r="I17">
-        <f t="shared" si="0"/>
-        <v>55.599999999999994</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+        <v>30.492651508586071</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>19</v>
       </c>
       <c r="B18">
-        <v>1.9321854999999999E-2</v>
+        <v>1.9731200000000001E-2</v>
       </c>
       <c r="C18">
         <v>10.7</v>
@@ -1174,20 +1049,15 @@
         <v>8.5500000000000007</v>
       </c>
       <c r="H18">
-        <f>AVERAGE(B18:D18,I18,G18)</f>
-        <v>132.74735599507522</v>
-      </c>
-      <c r="I18">
-        <f t="shared" si="0"/>
-        <v>551.15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+        <v>110.6228648867294</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>29</v>
       </c>
       <c r="B19">
-        <v>7.0799299999999999E-3</v>
+        <v>7.2904049999999998E-3</v>
       </c>
       <c r="C19">
         <v>10.7</v>
@@ -1205,20 +1075,15 @@
         <v>8.5500000000000007</v>
       </c>
       <c r="H19">
-        <f>AVERAGE(B19:D19,I19,G19)</f>
-        <v>134.08390609781426</v>
-      </c>
-      <c r="I19">
-        <f t="shared" si="0"/>
-        <v>558.6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+        <v>111.73662349401189</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>35</v>
       </c>
       <c r="B20">
-        <v>2.035992E-2</v>
+        <v>2.0623514999999999E-2</v>
       </c>
       <c r="C20">
         <v>10.25</v>
@@ -1236,20 +1101,15 @@
         <v>8.15</v>
       </c>
       <c r="H20">
-        <f>AVERAGE(B20:D20,I20,G20)</f>
-        <v>135.92582003552428</v>
-      </c>
-      <c r="I20">
-        <f t="shared" si="0"/>
-        <v>567.4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+        <v>113.2715606287702</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>45</v>
       </c>
       <c r="B21">
-        <v>7.6738649999999993E-3</v>
+        <v>8.0028149999999982E-3</v>
       </c>
       <c r="C21">
         <v>10.3</v>
@@ -1267,20 +1127,15 @@
         <v>8.15</v>
       </c>
       <c r="H21">
-        <f>AVERAGE(B21:D21,I21,G21)</f>
-        <v>137.61504880711917</v>
-      </c>
-      <c r="I21">
-        <f t="shared" si="0"/>
-        <v>576.6</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+        <v>114.67926216426589</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>49</v>
       </c>
       <c r="B22">
-        <v>2.3664145000000001E-2</v>
+        <v>2.4265624999999999E-2</v>
       </c>
       <c r="C22">
         <v>10.45</v>
@@ -1298,20 +1153,15 @@
         <v>8.4</v>
       </c>
       <c r="H22">
-        <f>AVERAGE(B22:D22,I22,G22)</f>
-        <v>144.69946108083383</v>
-      </c>
-      <c r="I22">
-        <f t="shared" si="0"/>
-        <v>611.25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+        <v>120.5829844806948</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>36</v>
       </c>
       <c r="B23">
-        <v>2.4732130000000001E-2</v>
+        <v>2.5352344999999998E-2</v>
       </c>
       <c r="C23">
         <v>10.7</v>
@@ -1329,20 +1179,15 @@
         <v>8.6999999999999993</v>
       </c>
       <c r="H23">
-        <f>AVERAGE(B23:D23,I23,G23)</f>
-        <v>147.3427479509453</v>
-      </c>
-      <c r="I23">
-        <f t="shared" si="0"/>
-        <v>623.65</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+        <v>122.7857266616211</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>15</v>
       </c>
       <c r="B24">
-        <v>6.7369350000000012E-3</v>
+        <v>6.9622649999999979E-3</v>
       </c>
       <c r="C24">
         <v>81.25</v>
@@ -1360,20 +1205,15 @@
         <v>14.8</v>
       </c>
       <c r="H24">
-        <f>AVERAGE(B24:D24,I24,G24)</f>
-        <v>150.40689354782549</v>
-      </c>
-      <c r="I24">
-        <f t="shared" si="0"/>
-        <v>558.6</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+        <v>125.3391155115212</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>10</v>
       </c>
       <c r="B25">
-        <v>1.9129275000000001E-2</v>
+        <v>1.9483629999999998E-2</v>
       </c>
       <c r="C25">
         <v>84.2</v>
@@ -1391,20 +1231,15 @@
         <v>18</v>
       </c>
       <c r="H25">
-        <f>AVERAGE(B25:D25,I25,G25)</f>
-        <v>150.41214330155077</v>
-      </c>
-      <c r="I25">
-        <f t="shared" si="0"/>
-        <v>551.15</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+        <v>125.34351181045901</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>20</v>
       </c>
       <c r="B26">
-        <v>1.9971699999999998E-2</v>
+        <v>2.0252124999999999E-2</v>
       </c>
       <c r="C26">
         <v>85.35</v>
@@ -1422,20 +1257,15 @@
         <v>14.4</v>
       </c>
       <c r="H26">
-        <f>AVERAGE(B26:D26,I26,G26)</f>
-        <v>153.33189548094731</v>
-      </c>
-      <c r="I26">
-        <f t="shared" si="0"/>
-        <v>567.4</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+        <v>127.7766263049561</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>30</v>
       </c>
       <c r="B27">
-        <v>7.3806150000000001E-3</v>
+        <v>7.6251099999999992E-3</v>
       </c>
       <c r="C27">
         <v>82.1</v>
@@ -1453,51 +1283,41 @@
         <v>13.4</v>
       </c>
       <c r="H27">
-        <f>AVERAGE(B27:D27,I27,G27)</f>
-        <v>153.98003743572716</v>
-      </c>
-      <c r="I27">
-        <f t="shared" si="0"/>
-        <v>576.6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="5" t="s">
+        <v>128.31673861227259</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="5">
-        <v>1.2139219999999999E-2</v>
-      </c>
-      <c r="C28" s="5">
+      <c r="B28">
+        <v>1.262339E-2</v>
+      </c>
+      <c r="C28">
         <v>10.65</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D28">
         <v>93.458215258242632</v>
       </c>
-      <c r="E28" s="5">
+      <c r="E28">
         <v>251.4</v>
       </c>
-      <c r="F28" s="5">
+      <c r="F28">
         <v>435.1</v>
       </c>
-      <c r="G28" s="5">
+      <c r="G28">
         <v>8.6</v>
       </c>
-      <c r="H28" s="5">
-        <f>AVERAGE(B28:D28,I28,G28)</f>
-        <v>159.84407089564854</v>
-      </c>
-      <c r="I28" s="5">
-        <f t="shared" si="0"/>
-        <v>686.5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H28">
+        <v>133.20347310804041</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>46</v>
       </c>
       <c r="B29">
-        <v>1.2880265E-2</v>
+        <v>1.325956E-2</v>
       </c>
       <c r="C29">
         <v>10.9</v>
@@ -1515,20 +1335,15 @@
         <v>8.9</v>
       </c>
       <c r="H29">
-        <f>AVERAGE(B29:D29,I29,G29)</f>
-        <v>160.48604923990703</v>
-      </c>
-      <c r="I29">
-        <f t="shared" si="0"/>
-        <v>688.8</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+        <v>133.73843758242251</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>37</v>
       </c>
       <c r="B30">
-        <v>2.3316819999999999E-2</v>
+        <v>2.4043615000000001E-2</v>
       </c>
       <c r="C30">
         <v>84</v>
@@ -1546,20 +1361,15 @@
         <v>14.35</v>
       </c>
       <c r="H30">
-        <f>AVERAGE(B30:D30,I30,G30)</f>
-        <v>161.56499091181851</v>
-      </c>
-      <c r="I30">
-        <f t="shared" si="0"/>
-        <v>611.25</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+        <v>134.63761355901539</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>21</v>
       </c>
       <c r="B31">
-        <v>2.4479785E-2</v>
+        <v>2.5071240000000002E-2</v>
       </c>
       <c r="C31">
         <v>84.8</v>
@@ -1577,20 +1387,15 @@
         <v>14.85</v>
       </c>
       <c r="H31">
-        <f>AVERAGE(B31:D31,I31,G31)</f>
-        <v>164.43208641982866</v>
-      </c>
-      <c r="I31">
-        <f t="shared" si="0"/>
-        <v>623.65</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+        <v>137.02683725902389</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>47</v>
       </c>
       <c r="B32">
-        <v>1.186721E-2</v>
+        <v>1.2266910000000001E-2</v>
       </c>
       <c r="C32">
         <v>83.7</v>
@@ -1608,20 +1413,15 @@
         <v>14.95</v>
       </c>
       <c r="H32">
-        <f>AVERAGE(B32:D32,I32,G32)</f>
-        <v>176.72039651603555</v>
-      </c>
-      <c r="I32">
-        <f t="shared" si="0"/>
-        <v>686.5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+        <v>147.26706371336289</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>31</v>
       </c>
       <c r="B33">
-        <v>1.2461885000000001E-2</v>
+        <v>1.2917339999999999E-2</v>
       </c>
       <c r="C33">
         <v>84.7</v>
@@ -1639,20 +1439,15 @@
         <v>15.35</v>
       </c>
       <c r="H33">
-        <f>AVERAGE(B33:D33,I33,G33)</f>
-        <v>177.56938846731344</v>
-      </c>
-      <c r="I33">
-        <f t="shared" si="0"/>
-        <v>688.8</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+        <v>147.97456629859451</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>32</v>
       </c>
       <c r="B34">
-        <v>7.4550449999999987E-3</v>
+        <v>7.688925000000001E-3</v>
       </c>
       <c r="C34">
         <v>11.35</v>
@@ -1670,20 +1465,15 @@
         <v>9.0500000000000007</v>
       </c>
       <c r="H34">
-        <f>AVERAGE(B34:D34,I34,G34)</f>
-        <v>239.72976701876823</v>
-      </c>
-      <c r="I34">
-        <f t="shared" si="0"/>
-        <v>1085.8</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+        <v>199.7748448289735</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>48</v>
       </c>
       <c r="B35">
-        <v>7.7811349999999998E-3</v>
+        <v>8.0742999999999995E-3</v>
       </c>
       <c r="C35">
         <v>11.3</v>
@@ -1701,20 +1491,15 @@
         <v>9.0500000000000007</v>
       </c>
       <c r="H35">
-        <f>AVERAGE(B35:D35,I35,G35)</f>
-        <v>241.85741230728348</v>
-      </c>
-      <c r="I35">
-        <f t="shared" si="0"/>
-        <v>1096.45</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+        <v>201.5478924502363</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>22</v>
       </c>
       <c r="B36">
-        <v>3.2635659999999997E-2</v>
+        <v>3.2938299999999997E-2</v>
       </c>
       <c r="C36">
         <v>10.1</v>
@@ -1732,20 +1517,15 @@
         <v>8.1</v>
       </c>
       <c r="H36">
-        <f>AVERAGE(B36:D36,I36,G36)</f>
-        <v>251.97822618782726</v>
-      </c>
-      <c r="I36">
-        <f t="shared" si="0"/>
-        <v>1151.3499999999999</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+        <v>209.98190559652281</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>16</v>
       </c>
       <c r="B37">
-        <v>7.1972900000000003E-3</v>
+        <v>7.4236899999999993E-3</v>
       </c>
       <c r="C37">
         <v>82.7</v>
@@ -1763,20 +1543,15 @@
         <v>16.25</v>
       </c>
       <c r="H37">
-        <f>AVERAGE(B37:D37,I37,G37)</f>
-        <v>256.43117826078804</v>
-      </c>
-      <c r="I37">
-        <f t="shared" si="0"/>
-        <v>1085.8</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+        <v>213.69268628399001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>38</v>
       </c>
       <c r="B38">
-        <v>3.1090300000000001E-2</v>
+        <v>3.1843799999999998E-2</v>
       </c>
       <c r="C38">
         <v>10.25</v>
@@ -1794,20 +1569,15 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="H38">
-        <f>AVERAGE(B38:D38,I38,G38)</f>
-        <v>257.82121636761673</v>
-      </c>
-      <c r="I38">
-        <f t="shared" si="0"/>
-        <v>1180.1500000000001</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+        <v>214.85113922301389</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>33</v>
       </c>
       <c r="B39">
-        <v>7.5326649999999992E-3</v>
+        <v>7.6831349999999989E-3</v>
       </c>
       <c r="C39">
         <v>82.9</v>
@@ -1825,20 +1595,15 @@
         <v>16.350000000000001</v>
       </c>
       <c r="H39">
-        <f>AVERAGE(B39:D39,I39,G39)</f>
-        <v>258.66952960703554</v>
-      </c>
-      <c r="I39">
-        <f t="shared" si="0"/>
-        <v>1096.45</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+        <v>215.5579664175296</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>11</v>
       </c>
       <c r="B40">
-        <v>3.2363935000000003E-2</v>
+        <v>3.2525424999999997E-2</v>
       </c>
       <c r="C40">
         <v>78.75</v>
@@ -1856,20 +1621,15 @@
         <v>11.75</v>
       </c>
       <c r="H40">
-        <f>AVERAGE(B40:D40,I40,G40)</f>
-        <v>267.29402904909324</v>
-      </c>
-      <c r="I40">
-        <f t="shared" si="0"/>
-        <v>1151.3499999999999</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+        <v>222.74505112257771</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>23</v>
       </c>
       <c r="B41">
-        <v>3.0958969999999999E-2</v>
+        <v>3.1391444999999997E-2</v>
       </c>
       <c r="C41">
         <v>79.05</v>
@@ -1887,20 +1647,15 @@
         <v>11.95</v>
       </c>
       <c r="H41">
-        <f>AVERAGE(B41:D41,I41,G41)</f>
-        <v>273.1888952423509</v>
-      </c>
-      <c r="I41">
-        <f t="shared" si="0"/>
-        <v>1180.1500000000001</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+        <v>227.6574847811257</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>34</v>
       </c>
       <c r="B42">
-        <v>6.7585299999999996E-3</v>
+        <v>7.006130000000001E-3</v>
       </c>
       <c r="C42">
         <v>9.75</v>
@@ -1918,20 +1673,15 @@
         <v>7.65</v>
       </c>
       <c r="H42">
-        <f>AVERAGE(B42:D42,I42,G42)</f>
-        <v>279.52907338096412</v>
-      </c>
-      <c r="I42">
-        <f t="shared" si="0"/>
-        <v>1289</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+        <v>232.94093575080339</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>18</v>
       </c>
       <c r="B43">
-        <v>6.4922350000000007E-3</v>
+        <v>6.6165349999999998E-3</v>
       </c>
       <c r="C43">
         <v>78.75</v>
@@ -1949,20 +1699,15 @@
         <v>12.3</v>
       </c>
       <c r="H43">
-        <f>AVERAGE(B43:D43,I43,G43)</f>
-        <v>295.01998169281535</v>
-      </c>
-      <c r="I43">
-        <f t="shared" si="0"/>
-        <v>1289</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+        <v>245.8500054606794</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>17</v>
       </c>
       <c r="B44">
-        <v>6.3105100000000001E-3</v>
+        <v>6.5135499999999999E-3</v>
       </c>
       <c r="C44">
         <v>9.65</v>
@@ -1980,20 +1725,15 @@
         <v>7.5</v>
       </c>
       <c r="H44">
-        <f>AVERAGE(B44:D44,I44,G44)</f>
-        <v>298.32732709869555</v>
-      </c>
-      <c r="I44">
-        <f t="shared" si="0"/>
-        <v>1383.5</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+        <v>248.60613975557959</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>9</v>
       </c>
       <c r="B45">
-        <v>6.0443949999999993E-3</v>
+        <v>6.2904950000000001E-3</v>
       </c>
       <c r="C45">
         <v>78.75</v>
@@ -2011,20 +1751,15 @@
         <v>12.65</v>
       </c>
       <c r="H45">
-        <f>AVERAGE(B45:D45,I45,G45)</f>
-        <v>314.00646066731031</v>
-      </c>
-      <c r="I45">
-        <f t="shared" si="0"/>
-        <v>1383.5</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+        <v>261.67209157275857</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>28</v>
       </c>
       <c r="B46">
-        <v>5.1722694999999999E-2</v>
+        <v>5.2772720000000002E-2</v>
       </c>
       <c r="C46">
         <v>9.25</v>
@@ -2042,20 +1777,15 @@
         <v>7.2</v>
       </c>
       <c r="H46">
-        <f>AVERAGE(B46:D46,I46,G46)</f>
-        <v>361.87680312098877</v>
-      </c>
-      <c r="I46">
-        <f t="shared" si="0"/>
-        <v>1701.45</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+        <v>301.56417760499068</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>13</v>
       </c>
       <c r="B47">
-        <v>5.3876260000000002E-2</v>
+        <v>5.4890015E-2</v>
       </c>
       <c r="C47">
         <v>9.1999999999999993</v>
@@ -2073,20 +1803,15 @@
         <v>7.2</v>
       </c>
       <c r="H47">
-        <f>AVERAGE(B47:D47,I47,G47)</f>
-        <v>362.35256829458797</v>
-      </c>
-      <c r="I47">
-        <f t="shared" si="0"/>
-        <v>1703.5</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+        <v>301.96064253798988</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>14</v>
       </c>
       <c r="B48">
-        <v>5.1545280000000013E-2</v>
+        <v>5.2416710000000012E-2</v>
       </c>
       <c r="C48">
         <v>78.75</v>
@@ -2104,20 +1829,15 @@
         <v>14.15</v>
       </c>
       <c r="H48">
-        <f>AVERAGE(B48:D48,I48,G48)</f>
-        <v>377.79786531809327</v>
-      </c>
-      <c r="I48">
-        <f t="shared" si="0"/>
-        <v>1701.45</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+        <v>314.83169967007768</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>8</v>
       </c>
       <c r="B49">
-        <v>5.3872875000000001E-2</v>
+        <v>5.4312930000000002E-2</v>
       </c>
       <c r="C49">
         <v>78.75</v>
@@ -2135,12 +1855,7 @@
         <v>17.95</v>
       </c>
       <c r="H49">
-        <f>AVERAGE(B49:D49,I49,G49)</f>
-        <v>378.96833083709328</v>
-      </c>
-      <c r="I49">
-        <f t="shared" si="0"/>
-        <v>1703.5</v>
+        <v>315.80701570674438</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
change the program of making map
</commit_message>
<xml_diff>
--- a/Excel/Rekap/Avg_Keseluruhan_All.xlsx
+++ b/Excel/Rekap/Avg_Keseluruhan_All.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEMHAS\TA_Python_Server\Excel\Rekap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0B7F1BB-7B1C-4BBE-9653-E74FBA8C5390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2838B567-7DCD-4BD1-A4CC-DF5AFB9C17E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$J$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$65</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -684,1206 +684,1206 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
-        <f t="shared" ref="A2:A33" si="0">LEN(B2)-LEN(SUBSTITUTE(B2,"-",""))+1</f>
-        <v>3</v>
+        <f>LEN(B2)-LEN(SUBSTITUTE(B2,"-",""))+1</f>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C2" s="2">
-        <v>2.9998849999999999E-3</v>
+        <v>6.9183300000000003E-3</v>
       </c>
       <c r="D2" s="2">
-        <v>21.25</v>
+        <v>43</v>
       </c>
       <c r="E2" s="2">
-        <v>7.1</v>
+        <v>8.9</v>
       </c>
       <c r="F2" s="2">
         <f>AVERAGE(C2:E2)</f>
-        <v>9.4509999616666676</v>
+        <v>17.30230611</v>
       </c>
       <c r="G2" s="2">
         <f>0.5*C2</f>
-        <v>1.4999424999999999E-3</v>
+        <v>3.4591650000000002E-3</v>
       </c>
       <c r="H2" s="2">
         <f>0.2*D2</f>
-        <v>4.25</v>
+        <v>8.6</v>
       </c>
       <c r="I2" s="2">
         <f>0.3*E2</f>
-        <v>2.13</v>
+        <v>2.67</v>
       </c>
       <c r="J2" s="2">
         <f>AVERAGE(G2:I2)</f>
-        <v>2.1271666474999997</v>
+        <v>3.7578197216666669</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>LEN(B3)-LEN(SUBSTITUTE(B3,"-",""))+1</f>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>59</v>
+        <v>7</v>
       </c>
       <c r="C3" s="2">
-        <v>3.3947049999999992E-3</v>
+        <v>4.5733000000000006E-3</v>
       </c>
       <c r="D3" s="2">
-        <v>24.05</v>
+        <v>144</v>
       </c>
       <c r="E3" s="2">
-        <v>7.2</v>
+        <v>13.25</v>
       </c>
       <c r="F3" s="2">
         <f>AVERAGE(C3:E3)</f>
-        <v>10.417798235000001</v>
+        <v>52.418191100000001</v>
       </c>
       <c r="G3" s="2">
         <f>0.5*C3</f>
-        <v>1.6973524999999996E-3</v>
+        <v>2.2866500000000003E-3</v>
       </c>
       <c r="H3" s="2">
         <f>0.2*D3</f>
-        <v>4.8100000000000005</v>
+        <v>28.8</v>
       </c>
       <c r="I3" s="2">
         <f>0.3*E3</f>
-        <v>2.16</v>
+        <v>3.9749999999999996</v>
       </c>
       <c r="J3" s="2">
         <f>AVERAGE(G3:I3)</f>
-        <v>2.3238991175000003</v>
+        <v>10.925762216666667</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
+        <f>LEN(B4)-LEN(SUBSTITUTE(B4,"-",""))+1</f>
+        <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="C4" s="2">
-        <v>2.99081E-3</v>
+        <v>3.4424345000000002E-2</v>
       </c>
       <c r="D4" s="2">
-        <v>21.25</v>
+        <v>899</v>
       </c>
       <c r="E4" s="2">
-        <v>10.4</v>
+        <v>11.75</v>
       </c>
       <c r="F4" s="2">
         <f>AVERAGE(C4:E4)</f>
-        <v>10.550996936666666</v>
+        <v>303.59480811500003</v>
       </c>
       <c r="G4" s="2">
         <f>0.5*C4</f>
-        <v>1.495405E-3</v>
+        <v>1.7212172500000001E-2</v>
       </c>
       <c r="H4" s="2">
         <f>0.2*D4</f>
-        <v>4.25</v>
+        <v>179.8</v>
       </c>
       <c r="I4" s="2">
         <f>0.3*E4</f>
-        <v>3.12</v>
+        <v>3.5249999999999999</v>
       </c>
       <c r="J4" s="2">
         <f>AVERAGE(G4:I4)</f>
-        <v>2.4571651349999999</v>
+        <v>61.114070724166673</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>LEN(B5)-LEN(SUBSTITUTE(B5,"-",""))+1</f>
+        <v>1</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="C5" s="2">
-        <v>4.0722349999999996E-3</v>
+        <v>6.3688800000000004E-3</v>
       </c>
       <c r="D5" s="2">
-        <v>24.75</v>
+        <v>1056.7</v>
       </c>
       <c r="E5" s="2">
-        <v>7.2</v>
+        <v>12.65</v>
       </c>
       <c r="F5" s="2">
         <f>AVERAGE(C5:E5)</f>
-        <v>10.651357411666666</v>
+        <v>356.45212296000005</v>
       </c>
       <c r="G5" s="2">
         <f>0.5*C5</f>
-        <v>2.0361174999999998E-3</v>
+        <v>3.1844400000000002E-3</v>
       </c>
       <c r="H5" s="2">
         <f>0.2*D5</f>
-        <v>4.95</v>
+        <v>211.34000000000003</v>
       </c>
       <c r="I5" s="2">
         <f>0.3*E5</f>
-        <v>2.16</v>
+        <v>3.7949999999999999</v>
       </c>
       <c r="J5" s="2">
         <f>AVERAGE(G5:I5)</f>
-        <v>2.3706787058333334</v>
+        <v>71.712728146666677</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>LEN(B6)-LEN(SUBSTITUTE(B6,"-",""))+1</f>
+        <v>1</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="C6" s="2">
-        <v>4.8914249999999996E-3</v>
+        <v>5.6884534999999993E-2</v>
       </c>
       <c r="D6" s="2">
-        <v>26.5</v>
+        <v>1440.25</v>
       </c>
       <c r="E6" s="2">
-        <v>5.75</v>
+        <v>5.25</v>
       </c>
       <c r="F6" s="2">
         <f>AVERAGE(C6:E6)</f>
-        <v>10.751630474999999</v>
+        <v>481.85229484500002</v>
       </c>
       <c r="G6" s="2">
         <f>0.5*C6</f>
-        <v>2.4457124999999998E-3</v>
+        <v>2.8442267499999997E-2</v>
       </c>
       <c r="H6" s="2">
         <f>0.2*D6</f>
-        <v>5.3000000000000007</v>
+        <v>288.05</v>
       </c>
       <c r="I6" s="2">
         <f>0.3*E6</f>
-        <v>1.7249999999999999</v>
+        <v>1.575</v>
       </c>
       <c r="J6" s="2">
         <f>AVERAGE(G6:I6)</f>
-        <v>2.3424819041666667</v>
+        <v>96.551147422499994</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f>LEN(B7)-LEN(SUBSTITUTE(B7,"-",""))+1</f>
+        <v>1</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="C7" s="2">
-        <v>3.3905149999999989E-3</v>
+        <v>5.6911955E-2</v>
       </c>
       <c r="D7" s="2">
-        <v>24.05</v>
+        <v>1440.25</v>
       </c>
       <c r="E7" s="2">
-        <v>10.25</v>
+        <v>17.95</v>
       </c>
       <c r="F7" s="2">
         <f>AVERAGE(C7:E7)</f>
-        <v>11.434463505000002</v>
+        <v>486.08563731833334</v>
       </c>
       <c r="G7" s="2">
         <f>0.5*C7</f>
-        <v>1.6952574999999994E-3</v>
+        <v>2.84559775E-2</v>
       </c>
       <c r="H7" s="2">
         <f>0.2*D7</f>
-        <v>4.8100000000000005</v>
+        <v>288.05</v>
       </c>
       <c r="I7" s="2">
         <f>0.3*E7</f>
-        <v>3.0749999999999997</v>
+        <v>5.3849999999999998</v>
       </c>
       <c r="J7" s="2">
         <f>AVERAGE(G7:I7)</f>
-        <v>2.6288984191666667</v>
+        <v>97.821151992500006</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <f>LEN(B8)-LEN(SUBSTITUTE(B8,"-",""))+1</f>
+        <v>1</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>63</v>
+        <v>11</v>
       </c>
       <c r="C8" s="2">
-        <v>5.2392799999999998E-3</v>
+        <v>5.5183359999999987E-2</v>
       </c>
       <c r="D8" s="2">
-        <v>28.45</v>
+        <v>1475.7</v>
       </c>
       <c r="E8" s="2">
-        <v>6.05</v>
+        <v>14.15</v>
       </c>
       <c r="F8" s="2">
         <f>AVERAGE(C8:E8)</f>
-        <v>11.501746426666665</v>
+        <v>496.63506112000005</v>
       </c>
       <c r="G8" s="2">
         <f>0.5*C8</f>
-        <v>2.6196399999999999E-3</v>
+        <v>2.7591679999999993E-2</v>
       </c>
       <c r="H8" s="2">
         <f>0.2*D8</f>
-        <v>5.69</v>
+        <v>295.14000000000004</v>
       </c>
       <c r="I8" s="2">
         <f>0.3*E8</f>
-        <v>1.8149999999999999</v>
+        <v>4.2450000000000001</v>
       </c>
       <c r="J8" s="2">
         <f>AVERAGE(G8:I8)</f>
-        <v>2.50253988</v>
+        <v>99.804197226666687</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <f>LEN(B9)-LEN(SUBSTITUTE(B9,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>67</v>
+        <v>22</v>
       </c>
       <c r="C9" s="2">
-        <v>5.5476900000000001E-3</v>
+        <v>2.99081E-3</v>
       </c>
       <c r="D9" s="2">
-        <v>28.25</v>
+        <v>21.25</v>
       </c>
       <c r="E9" s="2">
-        <v>6.25</v>
+        <v>10.4</v>
       </c>
       <c r="F9" s="2">
         <f>AVERAGE(C9:E9)</f>
-        <v>11.501849229999999</v>
+        <v>10.550996936666666</v>
       </c>
       <c r="G9" s="2">
         <f>0.5*C9</f>
-        <v>2.773845E-3</v>
+        <v>1.495405E-3</v>
       </c>
       <c r="H9" s="2">
         <f>0.2*D9</f>
-        <v>5.65</v>
+        <v>4.25</v>
       </c>
       <c r="I9" s="2">
         <f>0.3*E9</f>
-        <v>1.875</v>
+        <v>3.12</v>
       </c>
       <c r="J9" s="2">
         <f>AVERAGE(G9:I9)</f>
-        <v>2.5092579483333335</v>
+        <v>2.4571651349999999</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <f>LEN(B10)-LEN(SUBSTITUTE(B10,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C10" s="2">
-        <v>4.6681300000000004E-3</v>
+        <v>5.3853849999999986E-3</v>
       </c>
       <c r="D10" s="2">
-        <v>27.15</v>
+        <v>32.9</v>
       </c>
       <c r="E10" s="2">
-        <v>7.6</v>
+        <v>9.4</v>
       </c>
       <c r="F10" s="2">
         <f>AVERAGE(C10:E10)</f>
-        <v>11.584889376666666</v>
+        <v>14.101795128333331</v>
       </c>
       <c r="G10" s="2">
         <f>0.5*C10</f>
-        <v>2.3340650000000002E-3</v>
+        <v>2.6926924999999993E-3</v>
       </c>
       <c r="H10" s="2">
         <f>0.2*D10</f>
-        <v>5.43</v>
+        <v>6.58</v>
       </c>
       <c r="I10" s="2">
         <f>0.3*E10</f>
-        <v>2.2799999999999998</v>
+        <v>2.82</v>
       </c>
       <c r="J10" s="2">
         <f>AVERAGE(G10:I10)</f>
-        <v>2.5707780216666669</v>
+        <v>3.1342308975000002</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f>LEN(B11)-LEN(SUBSTITUTE(B11,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="C11" s="2">
-        <v>4.0778300000000002E-3</v>
+        <v>5.7008099999999997E-3</v>
       </c>
       <c r="D11" s="2">
-        <v>24.75</v>
+        <v>38.1</v>
       </c>
       <c r="E11" s="2">
-        <v>10.25</v>
+        <v>9.4</v>
       </c>
       <c r="F11" s="2">
         <f>AVERAGE(C11:E11)</f>
-        <v>11.668025943333333</v>
+        <v>15.835233603333334</v>
       </c>
       <c r="G11" s="2">
         <f>0.5*C11</f>
-        <v>2.0389150000000001E-3</v>
+        <v>2.8504049999999999E-3</v>
       </c>
       <c r="H11" s="2">
         <f>0.2*D11</f>
-        <v>4.95</v>
+        <v>7.620000000000001</v>
       </c>
       <c r="I11" s="2">
         <f>0.3*E11</f>
-        <v>3.0749999999999997</v>
+        <v>2.82</v>
       </c>
       <c r="J11" s="2">
         <f>AVERAGE(G11:I11)</f>
-        <v>2.6756796383333334</v>
+        <v>3.4809501350000005</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f>LEN(B12)-LEN(SUBSTITUTE(B12,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="C12" s="2">
-        <v>4.932225000000001E-3</v>
+        <v>6.8799050000000004E-3</v>
       </c>
       <c r="D12" s="2">
-        <v>26.5</v>
+        <v>43</v>
       </c>
       <c r="E12" s="2">
-        <v>8.8000000000000007</v>
+        <v>5.6</v>
       </c>
       <c r="F12" s="2">
         <f>AVERAGE(C12:E12)</f>
-        <v>11.768310741666667</v>
+        <v>16.202293301666668</v>
       </c>
       <c r="G12" s="2">
         <f>0.5*C12</f>
-        <v>2.4661125000000005E-3</v>
+        <v>3.4399525000000002E-3</v>
       </c>
       <c r="H12" s="2">
         <f>0.2*D12</f>
-        <v>5.3000000000000007</v>
+        <v>8.6</v>
       </c>
       <c r="I12" s="2">
         <f>0.3*E12</f>
-        <v>2.64</v>
+        <v>1.68</v>
       </c>
       <c r="J12" s="2">
         <f>AVERAGE(G12:I12)</f>
-        <v>2.6474887041666668</v>
+        <v>3.4278133175000001</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>LEN(B13)-LEN(SUBSTITUTE(B13,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="C13" s="2">
-        <v>5.2475600000000001E-3</v>
+        <v>1.1629415000000001E-2</v>
       </c>
       <c r="D13" s="2">
-        <v>28.45</v>
+        <v>62.2</v>
       </c>
       <c r="E13" s="2">
-        <v>9.25</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="F13" s="2">
         <f>AVERAGE(C13:E13)</f>
-        <v>12.568415853333335</v>
+        <v>23.803876471666669</v>
       </c>
       <c r="G13" s="2">
         <f>0.5*C13</f>
-        <v>2.62378E-3</v>
+        <v>5.8147075000000003E-3</v>
       </c>
       <c r="H13" s="2">
         <f>0.2*D13</f>
-        <v>5.69</v>
+        <v>12.440000000000001</v>
       </c>
       <c r="I13" s="2">
         <f>0.3*E13</f>
-        <v>2.7749999999999999</v>
+        <v>2.76</v>
       </c>
       <c r="J13" s="2">
         <f>AVERAGE(G13:I13)</f>
-        <v>2.8225412599999999</v>
+        <v>5.0686049025000006</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>LEN(B14)-LEN(SUBSTITUTE(B14,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="C14" s="2">
-        <v>5.5285949999999999E-3</v>
+        <v>4.5716250000000002E-3</v>
       </c>
       <c r="D14" s="2">
-        <v>28.25</v>
+        <v>144</v>
       </c>
       <c r="E14" s="2">
-        <v>9.4499999999999993</v>
+        <v>6.3</v>
       </c>
       <c r="F14" s="2">
         <f>AVERAGE(C14:E14)</f>
-        <v>12.568509531666669</v>
+        <v>50.101523875000005</v>
       </c>
       <c r="G14" s="2">
         <f>0.5*C14</f>
-        <v>2.7642974999999999E-3</v>
+        <v>2.2858125000000001E-3</v>
       </c>
       <c r="H14" s="2">
         <f>0.2*D14</f>
-        <v>5.65</v>
+        <v>28.8</v>
       </c>
       <c r="I14" s="2">
         <f>0.3*E14</f>
-        <v>2.8349999999999995</v>
+        <v>1.89</v>
       </c>
       <c r="J14" s="2">
         <f>AVERAGE(G14:I14)</f>
-        <v>2.8292547658333334</v>
+        <v>10.230761937500001</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
+        <f>LEN(B15)-LEN(SUBSTITUTE(B15,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="C15" s="2">
-        <v>5.9469650000000002E-3</v>
+        <v>4.7098149999999991E-3</v>
       </c>
       <c r="D15" s="2">
-        <v>31.1</v>
+        <v>144.44999999999999</v>
       </c>
       <c r="E15" s="2">
-        <v>6.9</v>
+        <v>11.25</v>
       </c>
       <c r="F15" s="2">
         <f>AVERAGE(C15:E15)</f>
-        <v>12.668648988333333</v>
+        <v>51.901569938333331</v>
       </c>
       <c r="G15" s="2">
         <f>0.5*C15</f>
-        <v>2.9734825000000001E-3</v>
+        <v>2.3549074999999996E-3</v>
       </c>
       <c r="H15" s="2">
         <f>0.2*D15</f>
-        <v>6.2200000000000006</v>
+        <v>28.89</v>
       </c>
       <c r="I15" s="2">
         <f>0.3*E15</f>
-        <v>2.0699999999999998</v>
+        <v>3.375</v>
       </c>
       <c r="J15" s="2">
         <f>AVERAGE(G15:I15)</f>
-        <v>2.7643244941666669</v>
+        <v>10.755784969166667</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>LEN(B16)-LEN(SUBSTITUTE(B16,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="C16" s="2">
-        <v>4.6912200000000003E-3</v>
+        <v>1.6257400000000001E-3</v>
       </c>
       <c r="D16" s="2">
-        <v>27.15</v>
+        <v>219.5</v>
       </c>
       <c r="E16" s="2">
-        <v>11</v>
+        <v>12.95</v>
       </c>
       <c r="F16" s="2">
         <f>AVERAGE(C16:E16)</f>
-        <v>12.718230406666668</v>
+        <v>77.48387524666667</v>
       </c>
       <c r="G16" s="2">
         <f>0.5*C16</f>
-        <v>2.3456100000000001E-3</v>
+        <v>8.1287000000000004E-4</v>
       </c>
       <c r="H16" s="2">
         <f>0.2*D16</f>
-        <v>5.43</v>
+        <v>43.900000000000006</v>
       </c>
       <c r="I16" s="2">
         <f>0.3*E16</f>
-        <v>3.3</v>
+        <v>3.8849999999999998</v>
       </c>
       <c r="J16" s="2">
         <f>AVERAGE(G16:I16)</f>
-        <v>2.9107818699999997</v>
+        <v>15.928604290000001</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f>LEN(B17)-LEN(SUBSTITUTE(B17,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="C17" s="2">
-        <v>5.3529099999999998E-3</v>
+        <v>7.6528249999999994E-3</v>
       </c>
       <c r="D17" s="2">
-        <v>32.9</v>
+        <v>236.9</v>
       </c>
       <c r="E17" s="2">
-        <v>6.7</v>
+        <v>21</v>
       </c>
       <c r="F17" s="2">
         <f>AVERAGE(C17:E17)</f>
-        <v>13.201784303333334</v>
+        <v>85.969217608333338</v>
       </c>
       <c r="G17" s="2">
         <f>0.5*C17</f>
-        <v>2.6764549999999999E-3</v>
+        <v>3.8264124999999997E-3</v>
       </c>
       <c r="H17" s="2">
         <f>0.2*D17</f>
-        <v>6.58</v>
+        <v>47.38</v>
       </c>
       <c r="I17" s="2">
         <f>0.3*E17</f>
-        <v>2.0099999999999998</v>
+        <v>6.3</v>
       </c>
       <c r="J17" s="2">
         <f>AVERAGE(G17:I17)</f>
-        <v>2.864225485</v>
+        <v>17.894608804166666</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <f>LEN(B18)-LEN(SUBSTITUTE(B18,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="C18" s="2">
-        <v>5.9296749999999997E-3</v>
+        <v>7.5226250000000007E-3</v>
       </c>
       <c r="D18" s="2">
-        <v>31.1</v>
+        <v>850.55</v>
       </c>
       <c r="E18" s="2">
-        <v>10.3</v>
+        <v>16.25</v>
       </c>
       <c r="F18" s="2">
         <f>AVERAGE(C18:E18)</f>
-        <v>13.801976558333335</v>
+        <v>288.935840875</v>
       </c>
       <c r="G18" s="2">
         <f>0.5*C18</f>
-        <v>2.9648374999999999E-3</v>
+        <v>3.7613125000000003E-3</v>
       </c>
       <c r="H18" s="2">
         <f>0.2*D18</f>
-        <v>6.2200000000000006</v>
+        <v>170.11</v>
       </c>
       <c r="I18" s="2">
         <f>0.3*E18</f>
-        <v>3.0900000000000003</v>
+        <v>4.875</v>
       </c>
       <c r="J18" s="2">
         <f>AVERAGE(G18:I18)</f>
-        <v>3.1043216125000002</v>
+        <v>58.32958710416667</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
-        <f t="shared" si="0"/>
+        <f>LEN(B19)-LEN(SUBSTITUTE(B19,"-",""))+1</f>
         <v>2</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C19" s="2">
-        <v>5.3853849999999986E-3</v>
+        <v>3.4309325000000002E-2</v>
       </c>
       <c r="D19" s="2">
-        <v>32.9</v>
+        <v>899</v>
       </c>
       <c r="E19" s="2">
-        <v>9.4</v>
+        <v>6.75</v>
       </c>
       <c r="F19" s="2">
         <f>AVERAGE(C19:E19)</f>
-        <v>14.101795128333331</v>
+        <v>301.92810310833335</v>
       </c>
       <c r="G19" s="2">
         <f>0.5*C19</f>
-        <v>2.6926924999999993E-3</v>
+        <v>1.7154662500000001E-2</v>
       </c>
       <c r="H19" s="2">
         <f>0.2*D19</f>
-        <v>6.58</v>
+        <v>179.8</v>
       </c>
       <c r="I19" s="2">
         <f>0.3*E19</f>
-        <v>2.82</v>
+        <v>2.0249999999999999</v>
       </c>
       <c r="J19" s="2">
         <f>AVERAGE(G19:I19)</f>
-        <v>3.1342308975000002</v>
+        <v>60.614051554166672</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <f>LEN(B20)-LEN(SUBSTITUTE(B20,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>66</v>
+        <v>20</v>
       </c>
       <c r="C20" s="2">
-        <v>6.3761149999999999E-3</v>
+        <v>3.2864059999999987E-2</v>
       </c>
       <c r="D20" s="2">
-        <v>35.65</v>
+        <v>909.1</v>
       </c>
       <c r="E20" s="2">
-        <v>7.3</v>
+        <v>11.95</v>
       </c>
       <c r="F20" s="2">
         <f>AVERAGE(C20:E20)</f>
-        <v>14.318792038333333</v>
+        <v>307.02762135333336</v>
       </c>
       <c r="G20" s="2">
         <f>0.5*C20</f>
-        <v>3.1880575E-3</v>
+        <v>1.6432029999999993E-2</v>
       </c>
       <c r="H20" s="2">
         <f>0.2*D20</f>
-        <v>7.13</v>
+        <v>181.82000000000002</v>
       </c>
       <c r="I20" s="2">
         <f>0.3*E20</f>
-        <v>2.19</v>
+        <v>3.5849999999999995</v>
       </c>
       <c r="J20" s="2">
         <f>AVERAGE(G20:I20)</f>
-        <v>3.1077293524999998</v>
+        <v>61.807144010000009</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>LEN(B21)-LEN(SUBSTITUTE(B21,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="C21" s="2">
-        <v>5.9995400000000003E-3</v>
+        <v>6.6849850000000001E-3</v>
       </c>
       <c r="D21" s="2">
-        <v>35.9</v>
+        <v>1027.3499999999999</v>
       </c>
       <c r="E21" s="2">
-        <v>7.45</v>
+        <v>12.45</v>
       </c>
       <c r="F21" s="2">
         <f>AVERAGE(C21:E21)</f>
-        <v>14.451999846666666</v>
+        <v>346.6022283283333</v>
       </c>
       <c r="G21" s="2">
         <f>0.5*C21</f>
-        <v>2.9997700000000001E-3</v>
+        <v>3.3424925E-3</v>
       </c>
       <c r="H21" s="2">
         <f>0.2*D21</f>
-        <v>7.18</v>
+        <v>205.47</v>
       </c>
       <c r="I21" s="2">
         <f>0.3*E21</f>
-        <v>2.2349999999999999</v>
+        <v>3.7349999999999994</v>
       </c>
       <c r="J21" s="2">
         <f>AVERAGE(G21:I21)</f>
-        <v>3.1393332566666667</v>
+        <v>69.736114164166665</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f>LEN(B22)-LEN(SUBSTITUTE(B22,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="C22" s="2">
-        <v>5.6903549999999994E-3</v>
+        <v>6.3507149999999998E-3</v>
       </c>
       <c r="D22" s="2">
-        <v>38.1</v>
+        <v>1056.7</v>
       </c>
       <c r="E22" s="2">
-        <v>5.95</v>
+        <v>6.15</v>
       </c>
       <c r="F22" s="2">
         <f>AVERAGE(C22:E22)</f>
-        <v>14.685230118333335</v>
+        <v>354.2854502383334</v>
       </c>
       <c r="G22" s="2">
         <f>0.5*C22</f>
-        <v>2.8451774999999997E-3</v>
+        <v>3.1753574999999999E-3</v>
       </c>
       <c r="H22" s="2">
         <f>0.2*D22</f>
-        <v>7.620000000000001</v>
+        <v>211.34000000000003</v>
       </c>
       <c r="I22" s="2">
         <f>0.3*E22</f>
-        <v>1.7849999999999999</v>
+        <v>1.845</v>
       </c>
       <c r="J22" s="2">
         <f>AVERAGE(G22:I22)</f>
-        <v>3.1359483925</v>
+        <v>71.062725119166672</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>LEN(B23)-LEN(SUBSTITUTE(B23,"-",""))+1</f>
+        <v>2</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="C23" s="2">
-        <v>6.5709999999999996E-3</v>
+        <v>5.5317085000000002E-2</v>
       </c>
       <c r="D23" s="2">
-        <v>38.75</v>
+        <v>1475.7</v>
       </c>
       <c r="E23" s="2">
-        <v>6.95</v>
+        <v>5.7</v>
       </c>
       <c r="F23" s="2">
         <f>AVERAGE(C23:E23)</f>
-        <v>15.235523666666667</v>
+        <v>493.81843902833339</v>
       </c>
       <c r="G23" s="2">
         <f>0.5*C23</f>
-        <v>3.2854999999999998E-3</v>
+        <v>2.7658542500000001E-2</v>
       </c>
       <c r="H23" s="2">
         <f>0.2*D23</f>
-        <v>7.75</v>
+        <v>295.14000000000004</v>
       </c>
       <c r="I23" s="2">
         <f>0.3*E23</f>
-        <v>2.085</v>
+        <v>1.71</v>
       </c>
       <c r="J23" s="2">
         <f>AVERAGE(G23:I23)</f>
-        <v>3.2794284999999999</v>
+        <v>98.959219514166662</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>LEN(B24)-LEN(SUBSTITUTE(B24,"-",""))+1</f>
+        <v>3</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="C24" s="2">
-        <v>6.3609700000000014E-3</v>
+        <v>2.9998849999999999E-3</v>
       </c>
       <c r="D24" s="2">
-        <v>35.65</v>
+        <v>21.25</v>
       </c>
       <c r="E24" s="2">
-        <v>11</v>
+        <v>7.1</v>
       </c>
       <c r="F24" s="2">
         <f>AVERAGE(C24:E24)</f>
-        <v>15.552120323333334</v>
+        <v>9.4509999616666676</v>
       </c>
       <c r="G24" s="2">
         <f>0.5*C24</f>
-        <v>3.1804850000000007E-3</v>
+        <v>1.4999424999999999E-3</v>
       </c>
       <c r="H24" s="2">
         <f>0.2*D24</f>
-        <v>7.13</v>
+        <v>4.25</v>
       </c>
       <c r="I24" s="2">
         <f>0.3*E24</f>
-        <v>3.3</v>
+        <v>2.13</v>
       </c>
       <c r="J24" s="2">
         <f>AVERAGE(G24:I24)</f>
-        <v>3.4777268283333331</v>
+        <v>2.1271666474999997</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
-        <f t="shared" si="0"/>
+        <f>LEN(B25)-LEN(SUBSTITUTE(B25,"-",""))+1</f>
         <v>3</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C25" s="2">
-        <v>6.0230149999999996E-3</v>
+        <v>3.3905149999999989E-3</v>
       </c>
       <c r="D25" s="2">
-        <v>35.9</v>
+        <v>24.05</v>
       </c>
       <c r="E25" s="2">
-        <v>11.05</v>
+        <v>10.25</v>
       </c>
       <c r="F25" s="2">
         <f>AVERAGE(C25:E25)</f>
-        <v>15.652007671666667</v>
+        <v>11.434463505000002</v>
       </c>
       <c r="G25" s="2">
         <f>0.5*C25</f>
-        <v>3.0115074999999998E-3</v>
+        <v>1.6952574999999994E-3</v>
       </c>
       <c r="H25" s="2">
         <f>0.2*D25</f>
-        <v>7.18</v>
+        <v>4.8100000000000005</v>
       </c>
       <c r="I25" s="2">
         <f>0.3*E25</f>
-        <v>3.3149999999999999</v>
+        <v>3.0749999999999997</v>
       </c>
       <c r="J25" s="2">
         <f>AVERAGE(G25:I25)</f>
-        <v>3.4993371691666666</v>
+        <v>2.6288984191666667</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
+        <f>LEN(B26)-LEN(SUBSTITUTE(B26,"-",""))+1</f>
+        <v>3</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="C26" s="2">
-        <v>5.7008099999999997E-3</v>
+        <v>4.0778300000000002E-3</v>
       </c>
       <c r="D26" s="2">
-        <v>38.1</v>
+        <v>24.75</v>
       </c>
       <c r="E26" s="2">
-        <v>9.4</v>
+        <v>10.25</v>
       </c>
       <c r="F26" s="2">
         <f>AVERAGE(C26:E26)</f>
-        <v>15.835233603333334</v>
+        <v>11.668025943333333</v>
       </c>
       <c r="G26" s="2">
         <f>0.5*C26</f>
-        <v>2.8504049999999999E-3</v>
+        <v>2.0389150000000001E-3</v>
       </c>
       <c r="H26" s="2">
         <f>0.2*D26</f>
-        <v>7.620000000000001</v>
+        <v>4.95</v>
       </c>
       <c r="I26" s="2">
         <f>0.3*E26</f>
-        <v>2.82</v>
+        <v>3.0749999999999997</v>
       </c>
       <c r="J26" s="2">
         <f>AVERAGE(G26:I26)</f>
-        <v>3.4809501350000005</v>
+        <v>2.6756796383333334</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
-        <f t="shared" si="0"/>
+        <f>LEN(B27)-LEN(SUBSTITUTE(B27,"-",""))+1</f>
         <v>3</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C27" s="2">
-        <v>6.5707200000000004E-3</v>
+        <v>4.932225000000001E-3</v>
       </c>
       <c r="D27" s="2">
-        <v>38.75</v>
+        <v>26.5</v>
       </c>
       <c r="E27" s="2">
-        <v>9.85</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="F27" s="2">
         <f>AVERAGE(C27:E27)</f>
-        <v>16.20219024</v>
+        <v>11.768310741666667</v>
       </c>
       <c r="G27" s="2">
         <f>0.5*C27</f>
-        <v>3.2853600000000002E-3</v>
+        <v>2.4661125000000005E-3</v>
       </c>
       <c r="H27" s="2">
         <f>0.2*D27</f>
-        <v>7.75</v>
+        <v>5.3000000000000007</v>
       </c>
       <c r="I27" s="2">
         <f>0.3*E27</f>
-        <v>2.9549999999999996</v>
+        <v>2.64</v>
       </c>
       <c r="J27" s="2">
         <f>AVERAGE(G27:I27)</f>
-        <v>3.5694284533333334</v>
+        <v>2.6474887041666668</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
+        <f>LEN(B28)-LEN(SUBSTITUTE(B28,"-",""))+1</f>
+        <v>3</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="C28" s="2">
-        <v>6.8799050000000004E-3</v>
+        <v>5.3529099999999998E-3</v>
       </c>
       <c r="D28" s="2">
-        <v>43</v>
+        <v>32.9</v>
       </c>
       <c r="E28" s="2">
-        <v>5.6</v>
+        <v>6.7</v>
       </c>
       <c r="F28" s="2">
         <f>AVERAGE(C28:E28)</f>
-        <v>16.202293301666668</v>
+        <v>13.201784303333334</v>
       </c>
       <c r="G28" s="2">
         <f>0.5*C28</f>
-        <v>3.4399525000000002E-3</v>
+        <v>2.6764549999999999E-3</v>
       </c>
       <c r="H28" s="2">
         <f>0.2*D28</f>
-        <v>8.6</v>
+        <v>6.58</v>
       </c>
       <c r="I28" s="2">
         <f>0.3*E28</f>
-        <v>1.68</v>
+        <v>2.0099999999999998</v>
       </c>
       <c r="J28" s="2">
         <f>AVERAGE(G28:I28)</f>
-        <v>3.4278133175000001</v>
+        <v>2.864225485</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>LEN(B29)-LEN(SUBSTITUTE(B29,"-",""))+1</f>
+        <v>3</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="C29" s="2">
-        <v>6.9183300000000003E-3</v>
+        <v>5.6903549999999994E-3</v>
       </c>
       <c r="D29" s="2">
-        <v>43</v>
+        <v>38.1</v>
       </c>
       <c r="E29" s="2">
-        <v>8.9</v>
+        <v>5.95</v>
       </c>
       <c r="F29" s="2">
         <f>AVERAGE(C29:E29)</f>
-        <v>17.30230611</v>
+        <v>14.685230118333335</v>
       </c>
       <c r="G29" s="2">
         <f>0.5*C29</f>
-        <v>3.4591650000000002E-3</v>
+        <v>2.8451774999999997E-3</v>
       </c>
       <c r="H29" s="2">
         <f>0.2*D29</f>
-        <v>8.6</v>
+        <v>7.620000000000001</v>
       </c>
       <c r="I29" s="2">
         <f>0.3*E29</f>
-        <v>2.67</v>
+        <v>1.7849999999999999</v>
       </c>
       <c r="J29" s="2">
         <f>AVERAGE(G29:I29)</f>
-        <v>3.7578197216666669</v>
+        <v>3.1359483925</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>LEN(B30)-LEN(SUBSTITUTE(B30,"-",""))+1</f>
+        <v>3</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="C30" s="2">
-        <v>8.2305450000000006E-3</v>
+        <v>6.0230149999999996E-3</v>
       </c>
       <c r="D30" s="2">
-        <v>45.9</v>
+        <v>35.9</v>
       </c>
       <c r="E30" s="2">
-        <v>6.1</v>
+        <v>11.05</v>
       </c>
       <c r="F30" s="2">
         <f>AVERAGE(C30:E30)</f>
-        <v>17.336076848333335</v>
+        <v>15.652007671666667</v>
       </c>
       <c r="G30" s="2">
         <f>0.5*C30</f>
-        <v>4.1152725000000003E-3</v>
+        <v>3.0115074999999998E-3</v>
       </c>
       <c r="H30" s="2">
         <f>0.2*D30</f>
-        <v>9.18</v>
+        <v>7.18</v>
       </c>
       <c r="I30" s="2">
         <f>0.3*E30</f>
-        <v>1.8299999999999998</v>
+        <v>3.3149999999999999</v>
       </c>
       <c r="J30" s="2">
         <f>AVERAGE(G30:I30)</f>
-        <v>3.6713717574999998</v>
+        <v>3.4993371691666666</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
-        <f t="shared" si="0"/>
+        <f>LEN(B31)-LEN(SUBSTITUTE(B31,"-",""))+1</f>
         <v>3</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C31" s="2">
-        <v>8.2380949999999991E-3</v>
+        <v>6.5707200000000004E-3</v>
       </c>
       <c r="D31" s="2">
-        <v>45.9</v>
+        <v>38.75</v>
       </c>
       <c r="E31" s="2">
-        <v>9.5</v>
+        <v>9.85</v>
       </c>
       <c r="F31" s="2">
         <f>AVERAGE(C31:E31)</f>
-        <v>18.469412698333333</v>
+        <v>16.20219024</v>
       </c>
       <c r="G31" s="2">
         <f>0.5*C31</f>
-        <v>4.1190474999999995E-3</v>
+        <v>3.2853600000000002E-3</v>
       </c>
       <c r="H31" s="2">
         <f>0.2*D31</f>
-        <v>9.18</v>
+        <v>7.75</v>
       </c>
       <c r="I31" s="2">
         <f>0.3*E31</f>
-        <v>2.85</v>
+        <v>2.9549999999999996</v>
       </c>
       <c r="J31" s="2">
         <f>AVERAGE(G31:I31)</f>
-        <v>4.0113730158333327</v>
+        <v>3.5694284533333334</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
-        <f t="shared" si="0"/>
+        <f>LEN(B32)-LEN(SUBSTITUTE(B32,"-",""))+1</f>
         <v>3</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C32" s="2">
-        <v>1.1661204999999999E-2</v>
+        <v>8.2380949999999991E-3</v>
       </c>
       <c r="D32" s="2">
-        <v>62.2</v>
+        <v>45.9</v>
       </c>
       <c r="E32" s="2">
-        <v>5.95</v>
+        <v>9.5</v>
       </c>
       <c r="F32" s="2">
         <f>AVERAGE(C32:E32)</f>
-        <v>22.720553734999999</v>
+        <v>18.469412698333333</v>
       </c>
       <c r="G32" s="2">
         <f>0.5*C32</f>
-        <v>5.8306024999999996E-3</v>
+        <v>4.1190474999999995E-3</v>
       </c>
       <c r="H32" s="2">
         <f>0.2*D32</f>
-        <v>12.440000000000001</v>
+        <v>9.18</v>
       </c>
       <c r="I32" s="2">
         <f>0.3*E32</f>
-        <v>1.7849999999999999</v>
+        <v>2.85</v>
       </c>
       <c r="J32" s="2">
         <f>AVERAGE(G32:I32)</f>
-        <v>4.7436102008333334</v>
+        <v>4.0113730158333327</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
+        <f>LEN(B33)-LEN(SUBSTITUTE(B33,"-",""))+1</f>
+        <v>3</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="C33" s="2">
-        <v>1.1629415000000001E-2</v>
+        <v>1.1661204999999999E-2</v>
       </c>
       <c r="D33" s="2">
         <v>62.2</v>
       </c>
       <c r="E33" s="2">
-        <v>9.1999999999999993</v>
+        <v>5.95</v>
       </c>
       <c r="F33" s="2">
         <f>AVERAGE(C33:E33)</f>
-        <v>23.803876471666669</v>
+        <v>22.720553734999999</v>
       </c>
       <c r="G33" s="2">
         <f>0.5*C33</f>
-        <v>5.8147075000000003E-3</v>
+        <v>5.8306024999999996E-3</v>
       </c>
       <c r="H33" s="2">
         <f>0.2*D33</f>
@@ -1891,1233 +1891,1234 @@
       </c>
       <c r="I33" s="2">
         <f>0.3*E33</f>
-        <v>2.76</v>
+        <v>1.7849999999999999</v>
       </c>
       <c r="J33" s="2">
         <f>AVERAGE(G33:I33)</f>
-        <v>5.0686049025000006</v>
+        <v>4.7436102008333334</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
-        <f t="shared" ref="A34:A65" si="1">LEN(B34)-LEN(SUBSTITUTE(B34,"-",""))+1</f>
-        <v>2</v>
+        <f>LEN(B34)-LEN(SUBSTITUTE(B34,"-",""))+1</f>
+        <v>3</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="C34" s="2">
-        <v>4.5716250000000002E-3</v>
+        <v>4.7251800000000007E-3</v>
       </c>
       <c r="D34" s="2">
-        <v>144</v>
+        <v>144.44999999999999</v>
       </c>
       <c r="E34" s="2">
-        <v>6.3</v>
+        <v>6.25</v>
       </c>
       <c r="F34" s="2">
         <f>AVERAGE(C34:E34)</f>
-        <v>50.101523875000005</v>
+        <v>50.234908393333335</v>
       </c>
       <c r="G34" s="2">
         <f>0.5*C34</f>
-        <v>2.2858125000000001E-3</v>
+        <v>2.3625900000000003E-3</v>
       </c>
       <c r="H34" s="2">
         <f>0.2*D34</f>
-        <v>28.8</v>
+        <v>28.89</v>
       </c>
       <c r="I34" s="2">
         <f>0.3*E34</f>
-        <v>1.89</v>
+        <v>1.875</v>
       </c>
       <c r="J34" s="2">
         <f>AVERAGE(G34:I34)</f>
-        <v>10.230761937500001</v>
+        <v>10.255787530000001</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
-        <f t="shared" si="1"/>
+        <f>LEN(B35)-LEN(SUBSTITUTE(B35,"-",""))+1</f>
         <v>3</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C35" s="2">
-        <v>4.7251800000000007E-3</v>
+        <v>1.8579E-3</v>
       </c>
       <c r="D35" s="2">
-        <v>144.44999999999999</v>
+        <v>211</v>
       </c>
       <c r="E35" s="2">
-        <v>6.25</v>
+        <v>12.45</v>
       </c>
       <c r="F35" s="2">
         <f>AVERAGE(C35:E35)</f>
-        <v>50.234908393333335</v>
+        <v>74.483952633333331</v>
       </c>
       <c r="G35" s="2">
         <f>0.5*C35</f>
-        <v>2.3625900000000003E-3</v>
+        <v>9.2895E-4</v>
       </c>
       <c r="H35" s="2">
         <f>0.2*D35</f>
-        <v>28.89</v>
+        <v>42.2</v>
       </c>
       <c r="I35" s="2">
         <f>0.3*E35</f>
-        <v>1.875</v>
+        <v>3.7349999999999994</v>
       </c>
       <c r="J35" s="2">
         <f>AVERAGE(G35:I35)</f>
-        <v>10.255787530000001</v>
+        <v>15.311976316666668</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f>LEN(B36)-LEN(SUBSTITUTE(B36,"-",""))+1</f>
+        <v>3</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="C36" s="2">
-        <v>4.7098149999999991E-3</v>
+        <v>1.6394249999999999E-3</v>
       </c>
       <c r="D36" s="2">
-        <v>144.44999999999999</v>
+        <v>219.5</v>
       </c>
       <c r="E36" s="2">
-        <v>11.25</v>
+        <v>6.75</v>
       </c>
       <c r="F36" s="2">
         <f>AVERAGE(C36:E36)</f>
-        <v>51.901569938333331</v>
+        <v>75.417213141666664</v>
       </c>
       <c r="G36" s="2">
         <f>0.5*C36</f>
-        <v>2.3549074999999996E-3</v>
+        <v>8.1971249999999996E-4</v>
       </c>
       <c r="H36" s="2">
         <f>0.2*D36</f>
-        <v>28.89</v>
+        <v>43.900000000000006</v>
       </c>
       <c r="I36" s="2">
         <f>0.3*E36</f>
-        <v>3.375</v>
+        <v>2.0249999999999999</v>
       </c>
       <c r="J36" s="2">
         <f>AVERAGE(G36:I36)</f>
-        <v>10.755784969166667</v>
+        <v>15.308606570833334</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f>LEN(B37)-LEN(SUBSTITUTE(B37,"-",""))+1</f>
+        <v>3</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C37" s="2">
+        <v>7.6514749999999996E-3</v>
+      </c>
+      <c r="D37" s="2">
+        <v>236.9</v>
+      </c>
+      <c r="E37" s="2">
         <v>7</v>
-      </c>
-      <c r="C37" s="2">
-        <v>4.5733000000000006E-3</v>
-      </c>
-      <c r="D37" s="2">
-        <v>144</v>
-      </c>
-      <c r="E37" s="2">
-        <v>13.25</v>
       </c>
       <c r="F37" s="2">
         <f>AVERAGE(C37:E37)</f>
-        <v>52.418191100000001</v>
+        <v>81.302550491666665</v>
       </c>
       <c r="G37" s="2">
         <f>0.5*C37</f>
-        <v>2.2866500000000003E-3</v>
+        <v>3.8257374999999998E-3</v>
       </c>
       <c r="H37" s="2">
         <f>0.2*D37</f>
-        <v>28.8</v>
+        <v>47.38</v>
       </c>
       <c r="I37" s="2">
         <f>0.3*E37</f>
-        <v>3.9749999999999996</v>
+        <v>2.1</v>
       </c>
       <c r="J37" s="2">
         <f>AVERAGE(G37:I37)</f>
-        <v>10.925762216666667</v>
+        <v>16.49460857916667</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
-        <f t="shared" si="1"/>
-        <v>4</v>
+        <f>LEN(B38)-LEN(SUBSTITUTE(B38,"-",""))+1</f>
+        <v>3</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="C38" s="2">
-        <v>1.854285E-3</v>
+        <v>8.0256600000000004E-3</v>
       </c>
       <c r="D38" s="2">
-        <v>211</v>
+        <v>241.7</v>
       </c>
       <c r="E38" s="2">
-        <v>6.65</v>
+        <v>11.55</v>
       </c>
       <c r="F38" s="2">
         <f>AVERAGE(C38:E38)</f>
-        <v>72.550618095000004</v>
+        <v>84.419341886666658</v>
       </c>
       <c r="G38" s="2">
         <f>0.5*C38</f>
-        <v>9.271425E-4</v>
+        <v>4.0128300000000002E-3</v>
       </c>
       <c r="H38" s="2">
         <f>0.2*D38</f>
-        <v>42.2</v>
+        <v>48.34</v>
       </c>
       <c r="I38" s="2">
         <f>0.3*E38</f>
-        <v>1.9950000000000001</v>
+        <v>3.4650000000000003</v>
       </c>
       <c r="J38" s="2">
         <f>AVERAGE(G38:I38)</f>
-        <v>14.731975714166666</v>
+        <v>17.269670943333335</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
-        <f t="shared" si="1"/>
+        <f>LEN(B39)-LEN(SUBSTITUTE(B39,"-",""))+1</f>
         <v>3</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C39" s="2">
-        <v>1.8579E-3</v>
+        <v>2.74085E-3</v>
       </c>
       <c r="D39" s="2">
-        <v>211</v>
+        <v>320.3</v>
       </c>
       <c r="E39" s="2">
-        <v>12.45</v>
+        <v>15.8</v>
       </c>
       <c r="F39" s="2">
         <f>AVERAGE(C39:E39)</f>
-        <v>74.483952633333331</v>
+        <v>112.03424695000001</v>
       </c>
       <c r="G39" s="2">
         <f>0.5*C39</f>
-        <v>9.2895E-4</v>
+        <v>1.370425E-3</v>
       </c>
       <c r="H39" s="2">
         <f>0.2*D39</f>
-        <v>42.2</v>
+        <v>64.06</v>
       </c>
       <c r="I39" s="2">
         <f>0.3*E39</f>
-        <v>3.7349999999999994</v>
+        <v>4.74</v>
       </c>
       <c r="J39" s="2">
         <f>AVERAGE(G39:I39)</f>
-        <v>15.311976316666668</v>
+        <v>22.933790141666666</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
-        <f t="shared" si="1"/>
+        <f>LEN(B40)-LEN(SUBSTITUTE(B40,"-",""))+1</f>
         <v>3</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C40" s="2">
-        <v>1.6394249999999999E-3</v>
+        <v>7.5190049999999996E-3</v>
       </c>
       <c r="D40" s="2">
-        <v>219.5</v>
+        <v>850.55</v>
       </c>
       <c r="E40" s="2">
-        <v>6.75</v>
+        <v>7.8</v>
       </c>
       <c r="F40" s="2">
         <f>AVERAGE(C40:E40)</f>
-        <v>75.417213141666664</v>
+        <v>286.11917300166664</v>
       </c>
       <c r="G40" s="2">
         <f>0.5*C40</f>
-        <v>8.1971249999999996E-4</v>
+        <v>3.7595024999999998E-3</v>
       </c>
       <c r="H40" s="2">
         <f>0.2*D40</f>
-        <v>43.900000000000006</v>
+        <v>170.11</v>
       </c>
       <c r="I40" s="2">
         <f>0.3*E40</f>
-        <v>2.0249999999999999</v>
+        <v>2.34</v>
       </c>
       <c r="J40" s="2">
         <f>AVERAGE(G40:I40)</f>
-        <v>15.308606570833334</v>
+        <v>57.484586500833338</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f>LEN(B41)-LEN(SUBSTITUTE(B41,"-",""))+1</f>
+        <v>3</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C41" s="2">
-        <v>1.6257400000000001E-3</v>
+        <v>7.7312300000000004E-3</v>
       </c>
       <c r="D41" s="2">
-        <v>219.5</v>
+        <v>861.65</v>
       </c>
       <c r="E41" s="2">
-        <v>12.95</v>
+        <v>16.3</v>
       </c>
       <c r="F41" s="2">
         <f>AVERAGE(C41:E41)</f>
-        <v>77.48387524666667</v>
+        <v>292.65257707666666</v>
       </c>
       <c r="G41" s="2">
         <f>0.5*C41</f>
-        <v>8.1287000000000004E-4</v>
+        <v>3.8656150000000002E-3</v>
       </c>
       <c r="H41" s="2">
         <f>0.2*D41</f>
-        <v>43.900000000000006</v>
+        <v>172.33</v>
       </c>
       <c r="I41" s="2">
         <f>0.3*E41</f>
-        <v>3.8849999999999998</v>
+        <v>4.8899999999999997</v>
       </c>
       <c r="J41" s="2">
         <f>AVERAGE(G41:I41)</f>
-        <v>15.928604290000001</v>
+        <v>59.074621871666665</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
-        <f t="shared" si="1"/>
+        <f>LEN(B42)-LEN(SUBSTITUTE(B42,"-",""))+1</f>
         <v>3</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C42" s="2">
-        <v>7.6514749999999996E-3</v>
+        <v>3.2857854999999991E-2</v>
       </c>
       <c r="D42" s="2">
-        <v>236.9</v>
+        <v>909.1</v>
       </c>
       <c r="E42" s="2">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="F42" s="2">
         <f>AVERAGE(C42:E42)</f>
-        <v>81.302550491666665</v>
+        <v>305.34428595166668</v>
       </c>
       <c r="G42" s="2">
         <f>0.5*C42</f>
-        <v>3.8257374999999998E-3</v>
+        <v>1.6428927499999996E-2</v>
       </c>
       <c r="H42" s="2">
         <f>0.2*D42</f>
-        <v>47.38</v>
+        <v>181.82000000000002</v>
       </c>
       <c r="I42" s="2">
         <f>0.3*E42</f>
-        <v>2.1</v>
+        <v>2.0699999999999998</v>
       </c>
       <c r="J42" s="2">
         <f>AVERAGE(G42:I42)</f>
-        <v>16.49460857916667</v>
+        <v>61.302142975833334</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
-        <f t="shared" si="1"/>
-        <v>4</v>
+        <f>LEN(B43)-LEN(SUBSTITUTE(B43,"-",""))+1</f>
+        <v>3</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="C43" s="2">
-        <v>8.0429749999999991E-3</v>
+        <v>6.6669549999999996E-3</v>
       </c>
       <c r="D43" s="2">
-        <v>241.7</v>
+        <v>1027.3499999999999</v>
       </c>
       <c r="E43" s="2">
-        <v>6.65</v>
+        <v>6.05</v>
       </c>
       <c r="F43" s="2">
         <f>AVERAGE(C43:E43)</f>
-        <v>82.786014324999996</v>
+        <v>344.46888898499992</v>
       </c>
       <c r="G43" s="2">
         <f>0.5*C43</f>
-        <v>4.0214874999999995E-3</v>
+        <v>3.3334774999999998E-3</v>
       </c>
       <c r="H43" s="2">
         <f>0.2*D43</f>
-        <v>48.34</v>
+        <v>205.47</v>
       </c>
       <c r="I43" s="2">
         <f>0.3*E43</f>
-        <v>1.9950000000000001</v>
+        <v>1.8149999999999999</v>
       </c>
       <c r="J43" s="2">
         <f>AVERAGE(G43:I43)</f>
-        <v>16.779673829166665</v>
+        <v>69.096111159166668</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
-        <f t="shared" si="1"/>
-        <v>3</v>
+        <f>LEN(B44)-LEN(SUBSTITUTE(B44,"-",""))+1</f>
+        <v>4</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="C44" s="2">
-        <v>8.0256600000000004E-3</v>
+        <v>3.3947049999999992E-3</v>
       </c>
       <c r="D44" s="2">
-        <v>241.7</v>
+        <v>24.05</v>
       </c>
       <c r="E44" s="2">
-        <v>11.55</v>
+        <v>7.2</v>
       </c>
       <c r="F44" s="2">
         <f>AVERAGE(C44:E44)</f>
-        <v>84.419341886666658</v>
+        <v>10.417798235000001</v>
       </c>
       <c r="G44" s="2">
         <f>0.5*C44</f>
-        <v>4.0128300000000002E-3</v>
+        <v>1.6973524999999996E-3</v>
       </c>
       <c r="H44" s="2">
         <f>0.2*D44</f>
-        <v>48.34</v>
+        <v>4.8100000000000005</v>
       </c>
       <c r="I44" s="2">
         <f>0.3*E44</f>
-        <v>3.4650000000000003</v>
+        <v>2.16</v>
       </c>
       <c r="J44" s="2">
         <f>AVERAGE(G44:I44)</f>
-        <v>17.269670943333335</v>
+        <v>2.3238991175000003</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f>LEN(B45)-LEN(SUBSTITUTE(B45,"-",""))+1</f>
+        <v>4</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="C45" s="2">
-        <v>7.6528249999999994E-3</v>
+        <v>4.0722349999999996E-3</v>
       </c>
       <c r="D45" s="2">
-        <v>236.9</v>
+        <v>24.75</v>
       </c>
       <c r="E45" s="2">
-        <v>21</v>
+        <v>7.2</v>
       </c>
       <c r="F45" s="2">
         <f>AVERAGE(C45:E45)</f>
-        <v>85.969217608333338</v>
+        <v>10.651357411666666</v>
       </c>
       <c r="G45" s="2">
         <f>0.5*C45</f>
-        <v>3.8264124999999997E-3</v>
+        <v>2.0361174999999998E-3</v>
       </c>
       <c r="H45" s="2">
         <f>0.2*D45</f>
-        <v>47.38</v>
+        <v>4.95</v>
       </c>
       <c r="I45" s="2">
         <f>0.3*E45</f>
-        <v>6.3</v>
+        <v>2.16</v>
       </c>
       <c r="J45" s="2">
         <f>AVERAGE(G45:I45)</f>
-        <v>17.894608804166666</v>
+        <v>2.3706787058333334</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
-        <f t="shared" si="1"/>
-        <v>5</v>
+        <f>LEN(B46)-LEN(SUBSTITUTE(B46,"-",""))+1</f>
+        <v>4</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C46" s="2">
-        <v>3.02287E-3</v>
+        <v>4.8914249999999996E-3</v>
       </c>
       <c r="D46" s="2">
-        <v>310.25</v>
+        <v>26.5</v>
       </c>
       <c r="E46" s="2">
-        <v>7.05</v>
+        <v>5.75</v>
       </c>
       <c r="F46" s="2">
         <f>AVERAGE(C46:E46)</f>
-        <v>105.76767429</v>
+        <v>10.751630474999999</v>
       </c>
       <c r="G46" s="2">
         <f>0.5*C46</f>
-        <v>1.511435E-3</v>
+        <v>2.4457124999999998E-3</v>
       </c>
       <c r="H46" s="2">
         <f>0.2*D46</f>
-        <v>62.050000000000004</v>
+        <v>5.3000000000000007</v>
       </c>
       <c r="I46" s="2">
         <f>0.3*E46</f>
-        <v>2.1149999999999998</v>
+        <v>1.7249999999999999</v>
       </c>
       <c r="J46" s="2">
         <f>AVERAGE(G46:I46)</f>
-        <v>21.388837145</v>
+        <v>2.3424819041666667</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
-        <f t="shared" si="1"/>
+        <f>LEN(B47)-LEN(SUBSTITUTE(B47,"-",""))+1</f>
         <v>4</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C47" s="2">
-        <v>3.065394999999999E-3</v>
+        <v>5.2475600000000001E-3</v>
       </c>
       <c r="D47" s="2">
-        <v>310.25</v>
+        <v>28.45</v>
       </c>
       <c r="E47" s="2">
-        <v>11.8</v>
+        <v>9.25</v>
       </c>
       <c r="F47" s="2">
         <f>AVERAGE(C47:E47)</f>
-        <v>107.35102179833335</v>
+        <v>12.568415853333335</v>
       </c>
       <c r="G47" s="2">
         <f>0.5*C47</f>
-        <v>1.5326974999999995E-3</v>
+        <v>2.62378E-3</v>
       </c>
       <c r="H47" s="2">
         <f>0.2*D47</f>
-        <v>62.050000000000004</v>
+        <v>5.69</v>
       </c>
       <c r="I47" s="2">
         <f>0.3*E47</f>
-        <v>3.54</v>
+        <v>2.7749999999999999</v>
       </c>
       <c r="J47" s="2">
         <f>AVERAGE(G47:I47)</f>
-        <v>21.8638442325</v>
+        <v>2.8225412599999999</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
-        <f t="shared" si="1"/>
+        <f>LEN(B48)-LEN(SUBSTITUTE(B48,"-",""))+1</f>
         <v>4</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C48" s="2">
-        <v>2.7397150000000002E-3</v>
+        <v>5.5285949999999999E-3</v>
       </c>
       <c r="D48" s="2">
-        <v>320.3</v>
+        <v>28.25</v>
       </c>
       <c r="E48" s="2">
-        <v>6.9</v>
+        <v>9.4499999999999993</v>
       </c>
       <c r="F48" s="2">
         <f>AVERAGE(C48:E48)</f>
-        <v>109.067579905</v>
+        <v>12.568509531666669</v>
       </c>
       <c r="G48" s="2">
         <f>0.5*C48</f>
-        <v>1.3698575000000001E-3</v>
+        <v>2.7642974999999999E-3</v>
       </c>
       <c r="H48" s="2">
         <f>0.2*D48</f>
-        <v>64.06</v>
+        <v>5.65</v>
       </c>
       <c r="I48" s="2">
         <f>0.3*E48</f>
-        <v>2.0699999999999998</v>
+        <v>2.8349999999999995</v>
       </c>
       <c r="J48" s="2">
         <f>AVERAGE(G48:I48)</f>
-        <v>22.043789952499996</v>
+        <v>2.8292547658333334</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
-        <f t="shared" si="1"/>
-        <v>3</v>
+        <f>LEN(B49)-LEN(SUBSTITUTE(B49,"-",""))+1</f>
+        <v>4</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="C49" s="2">
-        <v>2.74085E-3</v>
+        <v>4.6912200000000003E-3</v>
       </c>
       <c r="D49" s="2">
-        <v>320.3</v>
+        <v>27.15</v>
       </c>
       <c r="E49" s="2">
-        <v>15.8</v>
+        <v>11</v>
       </c>
       <c r="F49" s="2">
         <f>AVERAGE(C49:E49)</f>
-        <v>112.03424695000001</v>
+        <v>12.718230406666668</v>
       </c>
       <c r="G49" s="2">
         <f>0.5*C49</f>
-        <v>1.370425E-3</v>
+        <v>2.3456100000000001E-3</v>
       </c>
       <c r="H49" s="2">
         <f>0.2*D49</f>
-        <v>64.06</v>
+        <v>5.43</v>
       </c>
       <c r="I49" s="2">
         <f>0.3*E49</f>
-        <v>4.74</v>
+        <v>3.3</v>
       </c>
       <c r="J49" s="2">
         <f>AVERAGE(G49:I49)</f>
-        <v>22.933790141666666</v>
+        <v>2.9107818699999997</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
-        <f t="shared" si="1"/>
-        <v>3</v>
+        <f>LEN(B50)-LEN(SUBSTITUTE(B50,"-",""))+1</f>
+        <v>4</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="C50" s="2">
-        <v>7.5190049999999996E-3</v>
+        <v>5.9995400000000003E-3</v>
       </c>
       <c r="D50" s="2">
-        <v>850.55</v>
+        <v>35.9</v>
       </c>
       <c r="E50" s="2">
-        <v>7.8</v>
+        <v>7.45</v>
       </c>
       <c r="F50" s="2">
         <f>AVERAGE(C50:E50)</f>
-        <v>286.11917300166664</v>
+        <v>14.451999846666666</v>
       </c>
       <c r="G50" s="2">
         <f>0.5*C50</f>
-        <v>3.7595024999999998E-3</v>
+        <v>2.9997700000000001E-3</v>
       </c>
       <c r="H50" s="2">
         <f>0.2*D50</f>
-        <v>170.11</v>
+        <v>7.18</v>
       </c>
       <c r="I50" s="2">
         <f>0.3*E50</f>
-        <v>2.34</v>
+        <v>2.2349999999999999</v>
       </c>
       <c r="J50" s="2">
         <f>AVERAGE(G50:I50)</f>
-        <v>57.484586500833338</v>
+        <v>3.1393332566666667</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f>LEN(B51)-LEN(SUBSTITUTE(B51,"-",""))+1</f>
+        <v>4</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="C51" s="2">
-        <v>7.5226250000000007E-3</v>
+        <v>6.5709999999999996E-3</v>
       </c>
       <c r="D51" s="2">
-        <v>850.55</v>
+        <v>38.75</v>
       </c>
       <c r="E51" s="2">
-        <v>16.25</v>
+        <v>6.95</v>
       </c>
       <c r="F51" s="2">
         <f>AVERAGE(C51:E51)</f>
-        <v>288.935840875</v>
+        <v>15.235523666666667</v>
       </c>
       <c r="G51" s="2">
         <f>0.5*C51</f>
-        <v>3.7613125000000003E-3</v>
+        <v>3.2854999999999998E-3</v>
       </c>
       <c r="H51" s="2">
         <f>0.2*D51</f>
-        <v>170.11</v>
+        <v>7.75</v>
       </c>
       <c r="I51" s="2">
         <f>0.3*E51</f>
-        <v>4.875</v>
+        <v>2.085</v>
       </c>
       <c r="J51" s="2">
         <f>AVERAGE(G51:I51)</f>
-        <v>58.32958710416667</v>
+        <v>3.2794284999999999</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
-        <f t="shared" si="1"/>
+        <f>LEN(B52)-LEN(SUBSTITUTE(B52,"-",""))+1</f>
         <v>4</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C52" s="2">
-        <v>7.7455200000000014E-3</v>
+        <v>6.3609700000000014E-3</v>
       </c>
       <c r="D52" s="2">
-        <v>861.65</v>
+        <v>35.65</v>
       </c>
       <c r="E52" s="2">
-        <v>7.8</v>
+        <v>11</v>
       </c>
       <c r="F52" s="2">
         <f>AVERAGE(C52:E52)</f>
-        <v>289.81924850666661</v>
+        <v>15.552120323333334</v>
       </c>
       <c r="G52" s="2">
         <f>0.5*C52</f>
-        <v>3.8727600000000007E-3</v>
+        <v>3.1804850000000007E-3</v>
       </c>
       <c r="H52" s="2">
         <f>0.2*D52</f>
-        <v>172.33</v>
+        <v>7.13</v>
       </c>
       <c r="I52" s="2">
         <f>0.3*E52</f>
-        <v>2.34</v>
+        <v>3.3</v>
       </c>
       <c r="J52" s="2">
         <f>AVERAGE(G52:I52)</f>
-        <v>58.224624253333339</v>
+        <v>3.4777268283333331</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
-        <f t="shared" si="1"/>
-        <v>3</v>
+        <f>LEN(B53)-LEN(SUBSTITUTE(B53,"-",""))+1</f>
+        <v>4</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="C53" s="2">
-        <v>7.7312300000000004E-3</v>
+        <v>8.2305450000000006E-3</v>
       </c>
       <c r="D53" s="2">
-        <v>861.65</v>
+        <v>45.9</v>
       </c>
       <c r="E53" s="2">
-        <v>16.3</v>
+        <v>6.1</v>
       </c>
       <c r="F53" s="2">
         <f>AVERAGE(C53:E53)</f>
-        <v>292.65257707666666</v>
+        <v>17.336076848333335</v>
       </c>
       <c r="G53" s="2">
         <f>0.5*C53</f>
-        <v>3.8656150000000002E-3</v>
+        <v>4.1152725000000003E-3</v>
       </c>
       <c r="H53" s="2">
         <f>0.2*D53</f>
-        <v>172.33</v>
+        <v>9.18</v>
       </c>
       <c r="I53" s="2">
         <f>0.3*E53</f>
-        <v>4.8899999999999997</v>
+        <v>1.8299999999999998</v>
       </c>
       <c r="J53" s="2">
         <f>AVERAGE(G53:I53)</f>
-        <v>59.074621871666665</v>
+        <v>3.6713717574999998</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f>LEN(B54)-LEN(SUBSTITUTE(B54,"-",""))+1</f>
+        <v>4</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="C54" s="2">
-        <v>3.4309325000000002E-2</v>
+        <v>1.854285E-3</v>
       </c>
       <c r="D54" s="2">
-        <v>899</v>
+        <v>211</v>
       </c>
       <c r="E54" s="2">
-        <v>6.75</v>
+        <v>6.65</v>
       </c>
       <c r="F54" s="2">
         <f>AVERAGE(C54:E54)</f>
-        <v>301.92810310833335</v>
+        <v>72.550618095000004</v>
       </c>
       <c r="G54" s="2">
         <f>0.5*C54</f>
-        <v>1.7154662500000001E-2</v>
+        <v>9.271425E-4</v>
       </c>
       <c r="H54" s="2">
         <f>0.2*D54</f>
-        <v>179.8</v>
+        <v>42.2</v>
       </c>
       <c r="I54" s="2">
         <f>0.3*E54</f>
-        <v>2.0249999999999999</v>
+        <v>1.9950000000000001</v>
       </c>
       <c r="J54" s="2">
         <f>AVERAGE(G54:I54)</f>
-        <v>60.614051554166672</v>
+        <v>14.731975714166666</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f>LEN(B55)-LEN(SUBSTITUTE(B55,"-",""))+1</f>
+        <v>4</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="C55" s="2">
-        <v>3.4424345000000002E-2</v>
+        <v>8.0429749999999991E-3</v>
       </c>
       <c r="D55" s="2">
-        <v>899</v>
+        <v>241.7</v>
       </c>
       <c r="E55" s="2">
-        <v>11.75</v>
+        <v>6.65</v>
       </c>
       <c r="F55" s="2">
         <f>AVERAGE(C55:E55)</f>
-        <v>303.59480811500003</v>
+        <v>82.786014324999996</v>
       </c>
       <c r="G55" s="2">
         <f>0.5*C55</f>
-        <v>1.7212172500000001E-2</v>
+        <v>4.0214874999999995E-3</v>
       </c>
       <c r="H55" s="2">
         <f>0.2*D55</f>
-        <v>179.8</v>
+        <v>48.34</v>
       </c>
       <c r="I55" s="2">
         <f>0.3*E55</f>
-        <v>3.5249999999999999</v>
+        <v>1.9950000000000001</v>
       </c>
       <c r="J55" s="2">
         <f>AVERAGE(G55:I55)</f>
-        <v>61.114070724166673</v>
+        <v>16.779673829166665</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
-        <f t="shared" si="1"/>
-        <v>3</v>
+        <f>LEN(B56)-LEN(SUBSTITUTE(B56,"-",""))+1</f>
+        <v>4</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C56" s="2">
-        <v>3.2857854999999991E-2</v>
+        <v>3.065394999999999E-3</v>
       </c>
       <c r="D56" s="2">
-        <v>909.1</v>
+        <v>310.25</v>
       </c>
       <c r="E56" s="2">
-        <v>6.9</v>
+        <v>11.8</v>
       </c>
       <c r="F56" s="2">
         <f>AVERAGE(C56:E56)</f>
-        <v>305.34428595166668</v>
+        <v>107.35102179833335</v>
       </c>
       <c r="G56" s="2">
         <f>0.5*C56</f>
-        <v>1.6428927499999996E-2</v>
+        <v>1.5326974999999995E-3</v>
       </c>
       <c r="H56" s="2">
         <f>0.2*D56</f>
-        <v>181.82000000000002</v>
+        <v>62.050000000000004</v>
       </c>
       <c r="I56" s="2">
         <f>0.3*E56</f>
-        <v>2.0699999999999998</v>
+        <v>3.54</v>
       </c>
       <c r="J56" s="2">
         <f>AVERAGE(G56:I56)</f>
-        <v>61.302142975833334</v>
+        <v>21.8638442325</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f>LEN(B57)-LEN(SUBSTITUTE(B57,"-",""))+1</f>
+        <v>4</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="C57" s="2">
-        <v>3.2864059999999987E-2</v>
+        <v>2.7397150000000002E-3</v>
       </c>
       <c r="D57" s="2">
-        <v>909.1</v>
+        <v>320.3</v>
       </c>
       <c r="E57" s="2">
-        <v>11.95</v>
+        <v>6.9</v>
       </c>
       <c r="F57" s="2">
         <f>AVERAGE(C57:E57)</f>
-        <v>307.02762135333336</v>
+        <v>109.067579905</v>
       </c>
       <c r="G57" s="2">
         <f>0.5*C57</f>
-        <v>1.6432029999999993E-2</v>
+        <v>1.3698575000000001E-3</v>
       </c>
       <c r="H57" s="2">
         <f>0.2*D57</f>
-        <v>181.82000000000002</v>
+        <v>64.06</v>
       </c>
       <c r="I57" s="2">
         <f>0.3*E57</f>
-        <v>3.5849999999999995</v>
+        <v>2.0699999999999998</v>
       </c>
       <c r="J57" s="2">
         <f>AVERAGE(G57:I57)</f>
-        <v>61.807144010000009</v>
+        <v>22.043789952499996</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
-        <f t="shared" si="1"/>
-        <v>3</v>
+        <f>LEN(B58)-LEN(SUBSTITUTE(B58,"-",""))+1</f>
+        <v>4</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="C58" s="2">
-        <v>6.6669549999999996E-3</v>
+        <v>7.7455200000000014E-3</v>
       </c>
       <c r="D58" s="2">
-        <v>1027.3499999999999</v>
+        <v>861.65</v>
       </c>
       <c r="E58" s="2">
-        <v>6.05</v>
+        <v>7.8</v>
       </c>
       <c r="F58" s="2">
         <f>AVERAGE(C58:E58)</f>
-        <v>344.46888898499992</v>
+        <v>289.81924850666661</v>
       </c>
       <c r="G58" s="2">
         <f>0.5*C58</f>
-        <v>3.3334774999999998E-3</v>
+        <v>3.8727600000000007E-3</v>
       </c>
       <c r="H58" s="2">
         <f>0.2*D58</f>
-        <v>205.47</v>
+        <v>172.33</v>
       </c>
       <c r="I58" s="2">
         <f>0.3*E58</f>
-        <v>1.8149999999999999</v>
+        <v>2.34</v>
       </c>
       <c r="J58" s="2">
         <f>AVERAGE(G58:I58)</f>
-        <v>69.096111159166668</v>
+        <v>58.224624253333339</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f>LEN(B59)-LEN(SUBSTITUTE(B59,"-",""))+1</f>
+        <v>5</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="C59" s="2">
-        <v>6.6849850000000001E-3</v>
+        <v>5.2392799999999998E-3</v>
       </c>
       <c r="D59" s="2">
-        <v>1027.3499999999999</v>
+        <v>28.45</v>
       </c>
       <c r="E59" s="2">
-        <v>12.45</v>
+        <v>6.05</v>
       </c>
       <c r="F59" s="2">
         <f>AVERAGE(C59:E59)</f>
-        <v>346.6022283283333</v>
+        <v>11.501746426666665</v>
       </c>
       <c r="G59" s="2">
         <f>0.5*C59</f>
-        <v>3.3424925E-3</v>
+        <v>2.6196399999999999E-3</v>
       </c>
       <c r="H59" s="2">
         <f>0.2*D59</f>
-        <v>205.47</v>
+        <v>5.69</v>
       </c>
       <c r="I59" s="2">
         <f>0.3*E59</f>
-        <v>3.7349999999999994</v>
+        <v>1.8149999999999999</v>
       </c>
       <c r="J59" s="2">
         <f>AVERAGE(G59:I59)</f>
-        <v>69.736114164166665</v>
+        <v>2.50253988</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f>LEN(B60)-LEN(SUBSTITUTE(B60,"-",""))+1</f>
+        <v>5</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>14</v>
+        <v>67</v>
       </c>
       <c r="C60" s="2">
-        <v>6.3507149999999998E-3</v>
+        <v>5.5476900000000001E-3</v>
       </c>
       <c r="D60" s="2">
-        <v>1056.7</v>
+        <v>28.25</v>
       </c>
       <c r="E60" s="2">
-        <v>6.15</v>
+        <v>6.25</v>
       </c>
       <c r="F60" s="2">
         <f>AVERAGE(C60:E60)</f>
-        <v>354.2854502383334</v>
+        <v>11.501849229999999</v>
       </c>
       <c r="G60" s="2">
         <f>0.5*C60</f>
-        <v>3.1753574999999999E-3</v>
+        <v>2.773845E-3</v>
       </c>
       <c r="H60" s="2">
         <f>0.2*D60</f>
-        <v>211.34000000000003</v>
+        <v>5.65</v>
       </c>
       <c r="I60" s="2">
         <f>0.3*E60</f>
-        <v>1.845</v>
+        <v>1.875</v>
       </c>
       <c r="J60" s="2">
         <f>AVERAGE(G60:I60)</f>
-        <v>71.062725119166672</v>
+        <v>2.5092579483333335</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f>LEN(B61)-LEN(SUBSTITUTE(B61,"-",""))+1</f>
+        <v>5</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>6</v>
+        <v>64</v>
       </c>
       <c r="C61" s="2">
-        <v>6.3688800000000004E-3</v>
+        <v>4.6681300000000004E-3</v>
       </c>
       <c r="D61" s="2">
-        <v>1056.7</v>
+        <v>27.15</v>
       </c>
       <c r="E61" s="2">
-        <v>12.65</v>
+        <v>7.6</v>
       </c>
       <c r="F61" s="2">
         <f>AVERAGE(C61:E61)</f>
-        <v>356.45212296000005</v>
+        <v>11.584889376666666</v>
       </c>
       <c r="G61" s="2">
         <f>0.5*C61</f>
-        <v>3.1844400000000002E-3</v>
+        <v>2.3340650000000002E-3</v>
       </c>
       <c r="H61" s="2">
         <f>0.2*D61</f>
-        <v>211.34000000000003</v>
+        <v>5.43</v>
       </c>
       <c r="I61" s="2">
         <f>0.3*E61</f>
-        <v>3.7949999999999999</v>
+        <v>2.2799999999999998</v>
       </c>
       <c r="J61" s="2">
         <f>AVERAGE(G61:I61)</f>
-        <v>71.712728146666677</v>
+        <v>2.5707780216666669</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f>LEN(B62)-LEN(SUBSTITUTE(B62,"-",""))+1</f>
+        <v>5</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="C62" s="2">
-        <v>5.6884534999999993E-2</v>
+        <v>5.9296749999999997E-3</v>
       </c>
       <c r="D62" s="2">
-        <v>1440.25</v>
+        <v>31.1</v>
       </c>
       <c r="E62" s="2">
-        <v>5.25</v>
+        <v>10.3</v>
       </c>
       <c r="F62" s="2">
         <f>AVERAGE(C62:E62)</f>
-        <v>481.85229484500002</v>
+        <v>13.801976558333335</v>
       </c>
       <c r="G62" s="2">
         <f>0.5*C62</f>
-        <v>2.8442267499999997E-2</v>
+        <v>2.9648374999999999E-3</v>
       </c>
       <c r="H62" s="2">
         <f>0.2*D62</f>
-        <v>288.05</v>
+        <v>6.2200000000000006</v>
       </c>
       <c r="I62" s="2">
         <f>0.3*E62</f>
-        <v>1.575</v>
+        <v>3.0900000000000003</v>
       </c>
       <c r="J62" s="2">
         <f>AVERAGE(G62:I62)</f>
-        <v>96.551147422499994</v>
+        <v>3.1043216125000002</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f>LEN(B63)-LEN(SUBSTITUTE(B63,"-",""))+1</f>
+        <v>5</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="C63" s="2">
-        <v>5.6911955E-2</v>
+        <v>6.3761149999999999E-3</v>
       </c>
       <c r="D63" s="2">
-        <v>1440.25</v>
+        <v>35.65</v>
       </c>
       <c r="E63" s="2">
-        <v>17.95</v>
+        <v>7.3</v>
       </c>
       <c r="F63" s="2">
         <f>AVERAGE(C63:E63)</f>
-        <v>486.08563731833334</v>
+        <v>14.318792038333333</v>
       </c>
       <c r="G63" s="2">
         <f>0.5*C63</f>
-        <v>2.84559775E-2</v>
+        <v>3.1880575E-3</v>
       </c>
       <c r="H63" s="2">
         <f>0.2*D63</f>
-        <v>288.05</v>
+        <v>7.13</v>
       </c>
       <c r="I63" s="2">
         <f>0.3*E63</f>
-        <v>5.3849999999999998</v>
+        <v>2.19</v>
       </c>
       <c r="J63" s="2">
         <f>AVERAGE(G63:I63)</f>
-        <v>97.821151992500006</v>
+        <v>3.1077293524999998</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f>LEN(B64)-LEN(SUBSTITUTE(B64,"-",""))+1</f>
+        <v>5</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="C64" s="2">
-        <v>5.5317085000000002E-2</v>
+        <v>3.02287E-3</v>
       </c>
       <c r="D64" s="2">
-        <v>1475.7</v>
+        <v>310.25</v>
       </c>
       <c r="E64" s="2">
-        <v>5.7</v>
+        <v>7.05</v>
       </c>
       <c r="F64" s="2">
         <f>AVERAGE(C64:E64)</f>
-        <v>493.81843902833339</v>
+        <v>105.76767429</v>
       </c>
       <c r="G64" s="2">
         <f>0.5*C64</f>
-        <v>2.7658542500000001E-2</v>
+        <v>1.511435E-3</v>
       </c>
       <c r="H64" s="2">
         <f>0.2*D64</f>
-        <v>295.14000000000004</v>
+        <v>62.050000000000004</v>
       </c>
       <c r="I64" s="2">
         <f>0.3*E64</f>
-        <v>1.71</v>
+        <v>2.1149999999999998</v>
       </c>
       <c r="J64" s="2">
         <f>AVERAGE(G64:I64)</f>
-        <v>98.959219514166662</v>
+        <v>21.388837145</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
-        <f t="shared" si="1"/>
-        <v>1</v>
+        <f>LEN(B65)-LEN(SUBSTITUTE(B65,"-",""))+1</f>
+        <v>6</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="C65" s="2">
-        <v>5.5183359999999987E-2</v>
+        <v>5.9469650000000002E-3</v>
       </c>
       <c r="D65" s="2">
-        <v>1475.7</v>
+        <v>31.1</v>
       </c>
       <c r="E65" s="2">
-        <v>14.15</v>
+        <v>6.9</v>
       </c>
       <c r="F65" s="2">
         <f>AVERAGE(C65:E65)</f>
-        <v>496.63506112000005</v>
+        <v>12.668648988333333</v>
       </c>
       <c r="G65" s="2">
         <f>0.5*C65</f>
-        <v>2.7591679999999993E-2</v>
+        <v>2.9734825000000001E-3</v>
       </c>
       <c r="H65" s="2">
         <f>0.2*D65</f>
-        <v>295.14000000000004</v>
+        <v>6.2200000000000006</v>
       </c>
       <c r="I65" s="2">
         <f>0.3*E65</f>
-        <v>4.2450000000000001</v>
+        <v>2.0699999999999998</v>
       </c>
       <c r="J65" s="2">
         <f>AVERAGE(G65:I65)</f>
-        <v>99.804197226666687</v>
+        <v>2.7643244941666669</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:J65" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:J65">
-      <sortCondition ref="F1:F65"/>
+  <autoFilter ref="A1:J65" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J65">
+      <sortCondition ref="A2:A65"/>
+      <sortCondition ref="F2:F65"/>
     </sortState>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J65">

</xml_diff>